<commit_message>
Map open top (OT) to 22UT/42UT; add 05/10/2026 data
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gate-move-summary.xlsx
+++ b/docs/gate-move-summary.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Compare" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daily Summary'!$A$1:$M$81</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'System Compare'!$A$1:$G$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daily Summary'!$A$1:$M$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'System Compare'!$A$1:$G$51</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M81"/>
+  <dimension ref="A1:M101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4422,8 +4422,988 @@
         <v>4</v>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>SMART BKK</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>BKK25</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Consignee</t>
+        </is>
+      </c>
+      <c r="F82" t="n">
+        <v>8</v>
+      </c>
+      <c r="G82" t="n">
+        <v>0</v>
+      </c>
+      <c r="H82" t="n">
+        <v>11</v>
+      </c>
+      <c r="I82" t="n">
+        <v>0</v>
+      </c>
+      <c r="J82" t="n">
+        <v>0</v>
+      </c>
+      <c r="K82" t="n">
+        <v>0</v>
+      </c>
+      <c r="L82" t="n">
+        <v>0</v>
+      </c>
+      <c r="M82" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>SMART BKK</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>BKK25</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F83" t="n">
+        <v>0</v>
+      </c>
+      <c r="G83" t="n">
+        <v>0</v>
+      </c>
+      <c r="H83" t="n">
+        <v>0</v>
+      </c>
+      <c r="I83" t="n">
+        <v>0</v>
+      </c>
+      <c r="J83" t="n">
+        <v>0</v>
+      </c>
+      <c r="K83" t="n">
+        <v>0</v>
+      </c>
+      <c r="L83" t="n">
+        <v>0</v>
+      </c>
+      <c r="M83" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>SMART BKK</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>BKK25</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Shipper</t>
+        </is>
+      </c>
+      <c r="F84" t="n">
+        <v>3</v>
+      </c>
+      <c r="G84" t="n">
+        <v>0</v>
+      </c>
+      <c r="H84" t="n">
+        <v>0</v>
+      </c>
+      <c r="I84" t="n">
+        <v>0</v>
+      </c>
+      <c r="J84" t="n">
+        <v>0</v>
+      </c>
+      <c r="K84" t="n">
+        <v>0</v>
+      </c>
+      <c r="L84" t="n">
+        <v>0</v>
+      </c>
+      <c r="M84" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>SMART BKK</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>BKK25</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F85" t="n">
+        <v>0</v>
+      </c>
+      <c r="G85" t="n">
+        <v>0</v>
+      </c>
+      <c r="H85" t="n">
+        <v>0</v>
+      </c>
+      <c r="I85" t="n">
+        <v>0</v>
+      </c>
+      <c r="J85" t="n">
+        <v>0</v>
+      </c>
+      <c r="K85" t="n">
+        <v>0</v>
+      </c>
+      <c r="L85" t="n">
+        <v>0</v>
+      </c>
+      <c r="M85" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>BKK27</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Consignee</t>
+        </is>
+      </c>
+      <c r="F86" t="n">
+        <v>9</v>
+      </c>
+      <c r="G86" t="n">
+        <v>0</v>
+      </c>
+      <c r="H86" t="n">
+        <v>13</v>
+      </c>
+      <c r="I86" t="n">
+        <v>0</v>
+      </c>
+      <c r="J86" t="n">
+        <v>0</v>
+      </c>
+      <c r="K86" t="n">
+        <v>0</v>
+      </c>
+      <c r="L86" t="n">
+        <v>0</v>
+      </c>
+      <c r="M86" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>BKK27</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F87" t="n">
+        <v>0</v>
+      </c>
+      <c r="G87" t="n">
+        <v>0</v>
+      </c>
+      <c r="H87" t="n">
+        <v>0</v>
+      </c>
+      <c r="I87" t="n">
+        <v>0</v>
+      </c>
+      <c r="J87" t="n">
+        <v>0</v>
+      </c>
+      <c r="K87" t="n">
+        <v>0</v>
+      </c>
+      <c r="L87" t="n">
+        <v>0</v>
+      </c>
+      <c r="M87" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>BKK27</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Shipper</t>
+        </is>
+      </c>
+      <c r="F88" t="n">
+        <v>9</v>
+      </c>
+      <c r="G88" t="n">
+        <v>0</v>
+      </c>
+      <c r="H88" t="n">
+        <v>12</v>
+      </c>
+      <c r="I88" t="n">
+        <v>1</v>
+      </c>
+      <c r="J88" t="n">
+        <v>1</v>
+      </c>
+      <c r="K88" t="n">
+        <v>0</v>
+      </c>
+      <c r="L88" t="n">
+        <v>0</v>
+      </c>
+      <c r="M88" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>BKK27</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F89" t="n">
+        <v>8</v>
+      </c>
+      <c r="G89" t="n">
+        <v>0</v>
+      </c>
+      <c r="H89" t="n">
+        <v>0</v>
+      </c>
+      <c r="I89" t="n">
+        <v>0</v>
+      </c>
+      <c r="J89" t="n">
+        <v>0</v>
+      </c>
+      <c r="K89" t="n">
+        <v>0</v>
+      </c>
+      <c r="L89" t="n">
+        <v>0</v>
+      </c>
+      <c r="M89" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>HAST</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>LCH27</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Consignee</t>
+        </is>
+      </c>
+      <c r="F90" t="n">
+        <v>8</v>
+      </c>
+      <c r="G90" t="n">
+        <v>0</v>
+      </c>
+      <c r="H90" t="n">
+        <v>8</v>
+      </c>
+      <c r="I90" t="n">
+        <v>0</v>
+      </c>
+      <c r="J90" t="n">
+        <v>2</v>
+      </c>
+      <c r="K90" t="n">
+        <v>0</v>
+      </c>
+      <c r="L90" t="n">
+        <v>0</v>
+      </c>
+      <c r="M90" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>HAST</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>LCH27</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F91" t="n">
+        <v>4</v>
+      </c>
+      <c r="G91" t="n">
+        <v>0</v>
+      </c>
+      <c r="H91" t="n">
+        <v>2</v>
+      </c>
+      <c r="I91" t="n">
+        <v>0</v>
+      </c>
+      <c r="J91" t="n">
+        <v>0</v>
+      </c>
+      <c r="K91" t="n">
+        <v>0</v>
+      </c>
+      <c r="L91" t="n">
+        <v>0</v>
+      </c>
+      <c r="M91" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>HAST</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>LCH27</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Shipper</t>
+        </is>
+      </c>
+      <c r="F92" t="n">
+        <v>14</v>
+      </c>
+      <c r="G92" t="n">
+        <v>0</v>
+      </c>
+      <c r="H92" t="n">
+        <v>1</v>
+      </c>
+      <c r="I92" t="n">
+        <v>0</v>
+      </c>
+      <c r="J92" t="n">
+        <v>2</v>
+      </c>
+      <c r="K92" t="n">
+        <v>0</v>
+      </c>
+      <c r="L92" t="n">
+        <v>0</v>
+      </c>
+      <c r="M92" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>HAST</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>LCH27</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F93" t="n">
+        <v>0</v>
+      </c>
+      <c r="G93" t="n">
+        <v>0</v>
+      </c>
+      <c r="H93" t="n">
+        <v>0</v>
+      </c>
+      <c r="I93" t="n">
+        <v>0</v>
+      </c>
+      <c r="J93" t="n">
+        <v>0</v>
+      </c>
+      <c r="K93" t="n">
+        <v>0</v>
+      </c>
+      <c r="L93" t="n">
+        <v>0</v>
+      </c>
+      <c r="M93" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>LCH28</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Consignee</t>
+        </is>
+      </c>
+      <c r="F94" t="n">
+        <v>0</v>
+      </c>
+      <c r="G94" t="n">
+        <v>0</v>
+      </c>
+      <c r="H94" t="n">
+        <v>2</v>
+      </c>
+      <c r="I94" t="n">
+        <v>0</v>
+      </c>
+      <c r="J94" t="n">
+        <v>0</v>
+      </c>
+      <c r="K94" t="n">
+        <v>0</v>
+      </c>
+      <c r="L94" t="n">
+        <v>0</v>
+      </c>
+      <c r="M94" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>LCH28</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F95" t="n">
+        <v>0</v>
+      </c>
+      <c r="G95" t="n">
+        <v>0</v>
+      </c>
+      <c r="H95" t="n">
+        <v>0</v>
+      </c>
+      <c r="I95" t="n">
+        <v>0</v>
+      </c>
+      <c r="J95" t="n">
+        <v>0</v>
+      </c>
+      <c r="K95" t="n">
+        <v>0</v>
+      </c>
+      <c r="L95" t="n">
+        <v>0</v>
+      </c>
+      <c r="M95" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>LCH28</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Shipper</t>
+        </is>
+      </c>
+      <c r="F96" t="n">
+        <v>3</v>
+      </c>
+      <c r="G96" t="n">
+        <v>0</v>
+      </c>
+      <c r="H96" t="n">
+        <v>0</v>
+      </c>
+      <c r="I96" t="n">
+        <v>0</v>
+      </c>
+      <c r="J96" t="n">
+        <v>0</v>
+      </c>
+      <c r="K96" t="n">
+        <v>0</v>
+      </c>
+      <c r="L96" t="n">
+        <v>0</v>
+      </c>
+      <c r="M96" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>LCH28</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F97" t="n">
+        <v>0</v>
+      </c>
+      <c r="G97" t="n">
+        <v>0</v>
+      </c>
+      <c r="H97" t="n">
+        <v>0</v>
+      </c>
+      <c r="I97" t="n">
+        <v>0</v>
+      </c>
+      <c r="J97" t="n">
+        <v>0</v>
+      </c>
+      <c r="K97" t="n">
+        <v>0</v>
+      </c>
+      <c r="L97" t="n">
+        <v>0</v>
+      </c>
+      <c r="M97" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Consignee</t>
+        </is>
+      </c>
+      <c r="F98" t="n">
+        <v>17</v>
+      </c>
+      <c r="G98" t="n">
+        <v>0</v>
+      </c>
+      <c r="H98" t="n">
+        <v>18</v>
+      </c>
+      <c r="I98" t="n">
+        <v>0</v>
+      </c>
+      <c r="J98" t="n">
+        <v>0</v>
+      </c>
+      <c r="K98" t="n">
+        <v>1</v>
+      </c>
+      <c r="L98" t="n">
+        <v>0</v>
+      </c>
+      <c r="M98" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F99" t="n">
+        <v>0</v>
+      </c>
+      <c r="G99" t="n">
+        <v>0</v>
+      </c>
+      <c r="H99" t="n">
+        <v>1</v>
+      </c>
+      <c r="I99" t="n">
+        <v>0</v>
+      </c>
+      <c r="J99" t="n">
+        <v>0</v>
+      </c>
+      <c r="K99" t="n">
+        <v>0</v>
+      </c>
+      <c r="L99" t="n">
+        <v>0</v>
+      </c>
+      <c r="M99" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Shipper</t>
+        </is>
+      </c>
+      <c r="F100" t="n">
+        <v>11</v>
+      </c>
+      <c r="G100" t="n">
+        <v>0</v>
+      </c>
+      <c r="H100" t="n">
+        <v>14</v>
+      </c>
+      <c r="I100" t="n">
+        <v>0</v>
+      </c>
+      <c r="J100" t="n">
+        <v>0</v>
+      </c>
+      <c r="K100" t="n">
+        <v>0</v>
+      </c>
+      <c r="L100" t="n">
+        <v>0</v>
+      </c>
+      <c r="M100" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F101" t="n">
+        <v>0</v>
+      </c>
+      <c r="G101" t="n">
+        <v>0</v>
+      </c>
+      <c r="H101" t="n">
+        <v>0</v>
+      </c>
+      <c r="I101" t="n">
+        <v>0</v>
+      </c>
+      <c r="J101" t="n">
+        <v>0</v>
+      </c>
+      <c r="K101" t="n">
+        <v>0</v>
+      </c>
+      <c r="L101" t="n">
+        <v>0</v>
+      </c>
+      <c r="M101" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M81"/>
+  <autoFilter ref="A1:M101"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4434,7 +5414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5634,8 +6614,298 @@
         <v>0</v>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>SMART BKK</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>BKK25</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>19</v>
+      </c>
+      <c r="F42" t="n">
+        <v>19</v>
+      </c>
+      <c r="G42" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>SMART BKK</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>BKK25</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>3</v>
+      </c>
+      <c r="F43" t="n">
+        <v>3</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>BKK27</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>22</v>
+      </c>
+      <c r="F44" t="n">
+        <v>22</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>BKK27</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>31</v>
+      </c>
+      <c r="F45" t="n">
+        <v>31</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>HAST</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>LCH27</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>24</v>
+      </c>
+      <c r="F46" t="n">
+        <v>24</v>
+      </c>
+      <c r="G46" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>HAST</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>LCH27</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>17</v>
+      </c>
+      <c r="F47" t="n">
+        <v>17</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>LCH28</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>2</v>
+      </c>
+      <c r="F48" t="n">
+        <v>2</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>LCH28</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>3</v>
+      </c>
+      <c r="F49" t="n">
+        <v>3</v>
+      </c>
+      <c r="G49" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>37</v>
+      </c>
+      <c r="F50" t="n">
+        <v>37</v>
+      </c>
+      <c r="G50" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>25</v>
+      </c>
+      <c r="F51" t="n">
+        <v>25</v>
+      </c>
+      <c r="G51" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G41"/>
+  <autoFilter ref="A1:G51"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Recognise 'OFF HIRE-…' job numbers; add 06/10/2026 data
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gate-move-summary.xlsx
+++ b/docs/gate-move-summary.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Compare" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daily Summary'!$A$1:$M$101</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'System Compare'!$A$1:$G$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daily Summary'!$A$1:$M$121</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'System Compare'!$A$1:$G$61</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M101"/>
+  <dimension ref="A1:M121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5402,8 +5402,988 @@
         <v>0</v>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>SMART BKK</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>BKK25</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Consignee</t>
+        </is>
+      </c>
+      <c r="F102" t="n">
+        <v>1</v>
+      </c>
+      <c r="G102" t="n">
+        <v>0</v>
+      </c>
+      <c r="H102" t="n">
+        <v>6</v>
+      </c>
+      <c r="I102" t="n">
+        <v>0</v>
+      </c>
+      <c r="J102" t="n">
+        <v>0</v>
+      </c>
+      <c r="K102" t="n">
+        <v>0</v>
+      </c>
+      <c r="L102" t="n">
+        <v>0</v>
+      </c>
+      <c r="M102" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>SMART BKK</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>BKK25</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F103" t="n">
+        <v>0</v>
+      </c>
+      <c r="G103" t="n">
+        <v>0</v>
+      </c>
+      <c r="H103" t="n">
+        <v>0</v>
+      </c>
+      <c r="I103" t="n">
+        <v>0</v>
+      </c>
+      <c r="J103" t="n">
+        <v>0</v>
+      </c>
+      <c r="K103" t="n">
+        <v>0</v>
+      </c>
+      <c r="L103" t="n">
+        <v>0</v>
+      </c>
+      <c r="M103" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>SMART BKK</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>BKK25</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Shipper</t>
+        </is>
+      </c>
+      <c r="F104" t="n">
+        <v>9</v>
+      </c>
+      <c r="G104" t="n">
+        <v>0</v>
+      </c>
+      <c r="H104" t="n">
+        <v>7</v>
+      </c>
+      <c r="I104" t="n">
+        <v>0</v>
+      </c>
+      <c r="J104" t="n">
+        <v>0</v>
+      </c>
+      <c r="K104" t="n">
+        <v>0</v>
+      </c>
+      <c r="L104" t="n">
+        <v>0</v>
+      </c>
+      <c r="M104" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>SMART BKK</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>BKK25</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F105" t="n">
+        <v>0</v>
+      </c>
+      <c r="G105" t="n">
+        <v>0</v>
+      </c>
+      <c r="H105" t="n">
+        <v>0</v>
+      </c>
+      <c r="I105" t="n">
+        <v>0</v>
+      </c>
+      <c r="J105" t="n">
+        <v>0</v>
+      </c>
+      <c r="K105" t="n">
+        <v>0</v>
+      </c>
+      <c r="L105" t="n">
+        <v>0</v>
+      </c>
+      <c r="M105" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>BKK27</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Consignee</t>
+        </is>
+      </c>
+      <c r="F106" t="n">
+        <v>21</v>
+      </c>
+      <c r="G106" t="n">
+        <v>0</v>
+      </c>
+      <c r="H106" t="n">
+        <v>19</v>
+      </c>
+      <c r="I106" t="n">
+        <v>2</v>
+      </c>
+      <c r="J106" t="n">
+        <v>2</v>
+      </c>
+      <c r="K106" t="n">
+        <v>0</v>
+      </c>
+      <c r="L106" t="n">
+        <v>0</v>
+      </c>
+      <c r="M106" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>BKK27</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F107" t="n">
+        <v>0</v>
+      </c>
+      <c r="G107" t="n">
+        <v>0</v>
+      </c>
+      <c r="H107" t="n">
+        <v>0</v>
+      </c>
+      <c r="I107" t="n">
+        <v>0</v>
+      </c>
+      <c r="J107" t="n">
+        <v>0</v>
+      </c>
+      <c r="K107" t="n">
+        <v>0</v>
+      </c>
+      <c r="L107" t="n">
+        <v>0</v>
+      </c>
+      <c r="M107" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>BKK27</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Shipper</t>
+        </is>
+      </c>
+      <c r="F108" t="n">
+        <v>9</v>
+      </c>
+      <c r="G108" t="n">
+        <v>0</v>
+      </c>
+      <c r="H108" t="n">
+        <v>12</v>
+      </c>
+      <c r="I108" t="n">
+        <v>0</v>
+      </c>
+      <c r="J108" t="n">
+        <v>1</v>
+      </c>
+      <c r="K108" t="n">
+        <v>0</v>
+      </c>
+      <c r="L108" t="n">
+        <v>0</v>
+      </c>
+      <c r="M108" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>BKK27</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F109" t="n">
+        <v>0</v>
+      </c>
+      <c r="G109" t="n">
+        <v>0</v>
+      </c>
+      <c r="H109" t="n">
+        <v>0</v>
+      </c>
+      <c r="I109" t="n">
+        <v>0</v>
+      </c>
+      <c r="J109" t="n">
+        <v>0</v>
+      </c>
+      <c r="K109" t="n">
+        <v>0</v>
+      </c>
+      <c r="L109" t="n">
+        <v>0</v>
+      </c>
+      <c r="M109" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>HAST</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>LCH27</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Consignee</t>
+        </is>
+      </c>
+      <c r="F110" t="n">
+        <v>3</v>
+      </c>
+      <c r="G110" t="n">
+        <v>0</v>
+      </c>
+      <c r="H110" t="n">
+        <v>9</v>
+      </c>
+      <c r="I110" t="n">
+        <v>0</v>
+      </c>
+      <c r="J110" t="n">
+        <v>10</v>
+      </c>
+      <c r="K110" t="n">
+        <v>0</v>
+      </c>
+      <c r="L110" t="n">
+        <v>0</v>
+      </c>
+      <c r="M110" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>HAST</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>LCH27</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F111" t="n">
+        <v>6</v>
+      </c>
+      <c r="G111" t="n">
+        <v>0</v>
+      </c>
+      <c r="H111" t="n">
+        <v>0</v>
+      </c>
+      <c r="I111" t="n">
+        <v>0</v>
+      </c>
+      <c r="J111" t="n">
+        <v>0</v>
+      </c>
+      <c r="K111" t="n">
+        <v>0</v>
+      </c>
+      <c r="L111" t="n">
+        <v>0</v>
+      </c>
+      <c r="M111" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>HAST</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>LCH27</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Shipper</t>
+        </is>
+      </c>
+      <c r="F112" t="n">
+        <v>12</v>
+      </c>
+      <c r="G112" t="n">
+        <v>0</v>
+      </c>
+      <c r="H112" t="n">
+        <v>1</v>
+      </c>
+      <c r="I112" t="n">
+        <v>0</v>
+      </c>
+      <c r="J112" t="n">
+        <v>2</v>
+      </c>
+      <c r="K112" t="n">
+        <v>0</v>
+      </c>
+      <c r="L112" t="n">
+        <v>0</v>
+      </c>
+      <c r="M112" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>HAST</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>LCH27</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F113" t="n">
+        <v>3</v>
+      </c>
+      <c r="G113" t="n">
+        <v>0</v>
+      </c>
+      <c r="H113" t="n">
+        <v>1</v>
+      </c>
+      <c r="I113" t="n">
+        <v>0</v>
+      </c>
+      <c r="J113" t="n">
+        <v>0</v>
+      </c>
+      <c r="K113" t="n">
+        <v>0</v>
+      </c>
+      <c r="L113" t="n">
+        <v>0</v>
+      </c>
+      <c r="M113" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>LCH28</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Consignee</t>
+        </is>
+      </c>
+      <c r="F114" t="n">
+        <v>0</v>
+      </c>
+      <c r="G114" t="n">
+        <v>0</v>
+      </c>
+      <c r="H114" t="n">
+        <v>1</v>
+      </c>
+      <c r="I114" t="n">
+        <v>0</v>
+      </c>
+      <c r="J114" t="n">
+        <v>0</v>
+      </c>
+      <c r="K114" t="n">
+        <v>0</v>
+      </c>
+      <c r="L114" t="n">
+        <v>0</v>
+      </c>
+      <c r="M114" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>LCH28</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F115" t="n">
+        <v>0</v>
+      </c>
+      <c r="G115" t="n">
+        <v>0</v>
+      </c>
+      <c r="H115" t="n">
+        <v>0</v>
+      </c>
+      <c r="I115" t="n">
+        <v>0</v>
+      </c>
+      <c r="J115" t="n">
+        <v>0</v>
+      </c>
+      <c r="K115" t="n">
+        <v>0</v>
+      </c>
+      <c r="L115" t="n">
+        <v>0</v>
+      </c>
+      <c r="M115" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>LCH28</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Shipper</t>
+        </is>
+      </c>
+      <c r="F116" t="n">
+        <v>0</v>
+      </c>
+      <c r="G116" t="n">
+        <v>0</v>
+      </c>
+      <c r="H116" t="n">
+        <v>0</v>
+      </c>
+      <c r="I116" t="n">
+        <v>0</v>
+      </c>
+      <c r="J116" t="n">
+        <v>0</v>
+      </c>
+      <c r="K116" t="n">
+        <v>0</v>
+      </c>
+      <c r="L116" t="n">
+        <v>0</v>
+      </c>
+      <c r="M116" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>LCH28</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F117" t="n">
+        <v>0</v>
+      </c>
+      <c r="G117" t="n">
+        <v>0</v>
+      </c>
+      <c r="H117" t="n">
+        <v>0</v>
+      </c>
+      <c r="I117" t="n">
+        <v>0</v>
+      </c>
+      <c r="J117" t="n">
+        <v>0</v>
+      </c>
+      <c r="K117" t="n">
+        <v>0</v>
+      </c>
+      <c r="L117" t="n">
+        <v>0</v>
+      </c>
+      <c r="M117" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Consignee</t>
+        </is>
+      </c>
+      <c r="F118" t="n">
+        <v>51</v>
+      </c>
+      <c r="G118" t="n">
+        <v>0</v>
+      </c>
+      <c r="H118" t="n">
+        <v>9</v>
+      </c>
+      <c r="I118" t="n">
+        <v>0</v>
+      </c>
+      <c r="J118" t="n">
+        <v>0</v>
+      </c>
+      <c r="K118" t="n">
+        <v>0</v>
+      </c>
+      <c r="L118" t="n">
+        <v>0</v>
+      </c>
+      <c r="M118" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F119" t="n">
+        <v>0</v>
+      </c>
+      <c r="G119" t="n">
+        <v>0</v>
+      </c>
+      <c r="H119" t="n">
+        <v>1</v>
+      </c>
+      <c r="I119" t="n">
+        <v>0</v>
+      </c>
+      <c r="J119" t="n">
+        <v>0</v>
+      </c>
+      <c r="K119" t="n">
+        <v>0</v>
+      </c>
+      <c r="L119" t="n">
+        <v>0</v>
+      </c>
+      <c r="M119" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Shipper</t>
+        </is>
+      </c>
+      <c r="F120" t="n">
+        <v>23</v>
+      </c>
+      <c r="G120" t="n">
+        <v>0</v>
+      </c>
+      <c r="H120" t="n">
+        <v>13</v>
+      </c>
+      <c r="I120" t="n">
+        <v>0</v>
+      </c>
+      <c r="J120" t="n">
+        <v>0</v>
+      </c>
+      <c r="K120" t="n">
+        <v>0</v>
+      </c>
+      <c r="L120" t="n">
+        <v>0</v>
+      </c>
+      <c r="M120" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F121" t="n">
+        <v>0</v>
+      </c>
+      <c r="G121" t="n">
+        <v>0</v>
+      </c>
+      <c r="H121" t="n">
+        <v>0</v>
+      </c>
+      <c r="I121" t="n">
+        <v>0</v>
+      </c>
+      <c r="J121" t="n">
+        <v>0</v>
+      </c>
+      <c r="K121" t="n">
+        <v>0</v>
+      </c>
+      <c r="L121" t="n">
+        <v>0</v>
+      </c>
+      <c r="M121" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M101"/>
+  <autoFilter ref="A1:M121"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5414,7 +6394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6904,8 +7884,298 @@
         <v>0</v>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>SMART BKK</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>BKK25</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>7</v>
+      </c>
+      <c r="F52" t="n">
+        <v>7</v>
+      </c>
+      <c r="G52" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>SMART BKK</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>BKK25</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>16</v>
+      </c>
+      <c r="F53" t="n">
+        <v>16</v>
+      </c>
+      <c r="G53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>BKK27</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>44</v>
+      </c>
+      <c r="F54" t="n">
+        <v>44</v>
+      </c>
+      <c r="G54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>BKK27</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>22</v>
+      </c>
+      <c r="F55" t="n">
+        <v>22</v>
+      </c>
+      <c r="G55" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>HAST</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>LCH27</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>28</v>
+      </c>
+      <c r="F56" t="n">
+        <v>28</v>
+      </c>
+      <c r="G56" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>HAST</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>LCH27</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>19</v>
+      </c>
+      <c r="F57" t="n">
+        <v>19</v>
+      </c>
+      <c r="G57" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>LCH28</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>1</v>
+      </c>
+      <c r="F58" t="n">
+        <v>1</v>
+      </c>
+      <c r="G58" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>LCH28</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>0</v>
+      </c>
+      <c r="F59" t="n">
+        <v>0</v>
+      </c>
+      <c r="G59" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>61</v>
+      </c>
+      <c r="F60" t="n">
+        <v>61</v>
+      </c>
+      <c r="G60" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>36</v>
+      </c>
+      <c r="F61" t="n">
+        <v>36</v>
+      </c>
+      <c r="G61" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G51"/>
+  <autoFilter ref="A1:G61"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Partial days: skip yards without reports; compare only locations in the system file; dd.mm.yy dates; add 08/10/2026
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gate-move-summary.xlsx
+++ b/docs/gate-move-summary.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Compare" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daily Summary'!$A$1:$M$141</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'System Compare'!$A$1:$G$71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daily Summary'!$A$1:$M$161</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'System Compare'!$A$1:$G$73</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M141"/>
+  <dimension ref="A1:M161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7362,8 +7362,988 @@
         <v>0</v>
       </c>
     </row>
+    <row r="142">
+      <c r="A142" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>SMART BKK</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>BKK25</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Consignee</t>
+        </is>
+      </c>
+      <c r="F142" t="n">
+        <v>2</v>
+      </c>
+      <c r="G142" t="n">
+        <v>0</v>
+      </c>
+      <c r="H142" t="n">
+        <v>3</v>
+      </c>
+      <c r="I142" t="n">
+        <v>0</v>
+      </c>
+      <c r="J142" t="n">
+        <v>0</v>
+      </c>
+      <c r="K142" t="n">
+        <v>0</v>
+      </c>
+      <c r="L142" t="n">
+        <v>0</v>
+      </c>
+      <c r="M142" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>SMART BKK</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>BKK25</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F143" t="n">
+        <v>0</v>
+      </c>
+      <c r="G143" t="n">
+        <v>0</v>
+      </c>
+      <c r="H143" t="n">
+        <v>0</v>
+      </c>
+      <c r="I143" t="n">
+        <v>0</v>
+      </c>
+      <c r="J143" t="n">
+        <v>0</v>
+      </c>
+      <c r="K143" t="n">
+        <v>0</v>
+      </c>
+      <c r="L143" t="n">
+        <v>0</v>
+      </c>
+      <c r="M143" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>SMART BKK</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>BKK25</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Shipper</t>
+        </is>
+      </c>
+      <c r="F144" t="n">
+        <v>6</v>
+      </c>
+      <c r="G144" t="n">
+        <v>0</v>
+      </c>
+      <c r="H144" t="n">
+        <v>5</v>
+      </c>
+      <c r="I144" t="n">
+        <v>0</v>
+      </c>
+      <c r="J144" t="n">
+        <v>0</v>
+      </c>
+      <c r="K144" t="n">
+        <v>0</v>
+      </c>
+      <c r="L144" t="n">
+        <v>0</v>
+      </c>
+      <c r="M144" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>SMART BKK</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>BKK25</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F145" t="n">
+        <v>0</v>
+      </c>
+      <c r="G145" t="n">
+        <v>0</v>
+      </c>
+      <c r="H145" t="n">
+        <v>0</v>
+      </c>
+      <c r="I145" t="n">
+        <v>0</v>
+      </c>
+      <c r="J145" t="n">
+        <v>0</v>
+      </c>
+      <c r="K145" t="n">
+        <v>0</v>
+      </c>
+      <c r="L145" t="n">
+        <v>0</v>
+      </c>
+      <c r="M145" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>BKK27</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Consignee</t>
+        </is>
+      </c>
+      <c r="F146" t="n">
+        <v>70</v>
+      </c>
+      <c r="G146" t="n">
+        <v>1</v>
+      </c>
+      <c r="H146" t="n">
+        <v>29</v>
+      </c>
+      <c r="I146" t="n">
+        <v>1</v>
+      </c>
+      <c r="J146" t="n">
+        <v>4</v>
+      </c>
+      <c r="K146" t="n">
+        <v>0</v>
+      </c>
+      <c r="L146" t="n">
+        <v>0</v>
+      </c>
+      <c r="M146" t="n">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>BKK27</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F147" t="n">
+        <v>0</v>
+      </c>
+      <c r="G147" t="n">
+        <v>0</v>
+      </c>
+      <c r="H147" t="n">
+        <v>0</v>
+      </c>
+      <c r="I147" t="n">
+        <v>0</v>
+      </c>
+      <c r="J147" t="n">
+        <v>0</v>
+      </c>
+      <c r="K147" t="n">
+        <v>0</v>
+      </c>
+      <c r="L147" t="n">
+        <v>0</v>
+      </c>
+      <c r="M147" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>BKK27</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Shipper</t>
+        </is>
+      </c>
+      <c r="F148" t="n">
+        <v>28</v>
+      </c>
+      <c r="G148" t="n">
+        <v>0</v>
+      </c>
+      <c r="H148" t="n">
+        <v>42</v>
+      </c>
+      <c r="I148" t="n">
+        <v>0</v>
+      </c>
+      <c r="J148" t="n">
+        <v>3</v>
+      </c>
+      <c r="K148" t="n">
+        <v>0</v>
+      </c>
+      <c r="L148" t="n">
+        <v>0</v>
+      </c>
+      <c r="M148" t="n">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>BKK27</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F149" t="n">
+        <v>0</v>
+      </c>
+      <c r="G149" t="n">
+        <v>0</v>
+      </c>
+      <c r="H149" t="n">
+        <v>0</v>
+      </c>
+      <c r="I149" t="n">
+        <v>0</v>
+      </c>
+      <c r="J149" t="n">
+        <v>0</v>
+      </c>
+      <c r="K149" t="n">
+        <v>0</v>
+      </c>
+      <c r="L149" t="n">
+        <v>0</v>
+      </c>
+      <c r="M149" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>HAST</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>LCH27</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>Consignee</t>
+        </is>
+      </c>
+      <c r="F150" t="n">
+        <v>4</v>
+      </c>
+      <c r="G150" t="n">
+        <v>0</v>
+      </c>
+      <c r="H150" t="n">
+        <v>13</v>
+      </c>
+      <c r="I150" t="n">
+        <v>0</v>
+      </c>
+      <c r="J150" t="n">
+        <v>6</v>
+      </c>
+      <c r="K150" t="n">
+        <v>0</v>
+      </c>
+      <c r="L150" t="n">
+        <v>0</v>
+      </c>
+      <c r="M150" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>HAST</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>LCH27</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F151" t="n">
+        <v>4</v>
+      </c>
+      <c r="G151" t="n">
+        <v>0</v>
+      </c>
+      <c r="H151" t="n">
+        <v>0</v>
+      </c>
+      <c r="I151" t="n">
+        <v>0</v>
+      </c>
+      <c r="J151" t="n">
+        <v>1</v>
+      </c>
+      <c r="K151" t="n">
+        <v>0</v>
+      </c>
+      <c r="L151" t="n">
+        <v>0</v>
+      </c>
+      <c r="M151" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>HAST</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>LCH27</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Shipper</t>
+        </is>
+      </c>
+      <c r="F152" t="n">
+        <v>5</v>
+      </c>
+      <c r="G152" t="n">
+        <v>0</v>
+      </c>
+      <c r="H152" t="n">
+        <v>5</v>
+      </c>
+      <c r="I152" t="n">
+        <v>0</v>
+      </c>
+      <c r="J152" t="n">
+        <v>6</v>
+      </c>
+      <c r="K152" t="n">
+        <v>0</v>
+      </c>
+      <c r="L152" t="n">
+        <v>0</v>
+      </c>
+      <c r="M152" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>HAST</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>LCH27</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F153" t="n">
+        <v>0</v>
+      </c>
+      <c r="G153" t="n">
+        <v>0</v>
+      </c>
+      <c r="H153" t="n">
+        <v>0</v>
+      </c>
+      <c r="I153" t="n">
+        <v>0</v>
+      </c>
+      <c r="J153" t="n">
+        <v>0</v>
+      </c>
+      <c r="K153" t="n">
+        <v>0</v>
+      </c>
+      <c r="L153" t="n">
+        <v>0</v>
+      </c>
+      <c r="M153" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>LCH28</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Consignee</t>
+        </is>
+      </c>
+      <c r="F154" t="n">
+        <v>0</v>
+      </c>
+      <c r="G154" t="n">
+        <v>0</v>
+      </c>
+      <c r="H154" t="n">
+        <v>1</v>
+      </c>
+      <c r="I154" t="n">
+        <v>0</v>
+      </c>
+      <c r="J154" t="n">
+        <v>0</v>
+      </c>
+      <c r="K154" t="n">
+        <v>0</v>
+      </c>
+      <c r="L154" t="n">
+        <v>0</v>
+      </c>
+      <c r="M154" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>LCH28</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F155" t="n">
+        <v>0</v>
+      </c>
+      <c r="G155" t="n">
+        <v>0</v>
+      </c>
+      <c r="H155" t="n">
+        <v>0</v>
+      </c>
+      <c r="I155" t="n">
+        <v>0</v>
+      </c>
+      <c r="J155" t="n">
+        <v>0</v>
+      </c>
+      <c r="K155" t="n">
+        <v>0</v>
+      </c>
+      <c r="L155" t="n">
+        <v>0</v>
+      </c>
+      <c r="M155" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>LCH28</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Shipper</t>
+        </is>
+      </c>
+      <c r="F156" t="n">
+        <v>0</v>
+      </c>
+      <c r="G156" t="n">
+        <v>0</v>
+      </c>
+      <c r="H156" t="n">
+        <v>0</v>
+      </c>
+      <c r="I156" t="n">
+        <v>0</v>
+      </c>
+      <c r="J156" t="n">
+        <v>0</v>
+      </c>
+      <c r="K156" t="n">
+        <v>0</v>
+      </c>
+      <c r="L156" t="n">
+        <v>0</v>
+      </c>
+      <c r="M156" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>LCH28</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F157" t="n">
+        <v>0</v>
+      </c>
+      <c r="G157" t="n">
+        <v>0</v>
+      </c>
+      <c r="H157" t="n">
+        <v>0</v>
+      </c>
+      <c r="I157" t="n">
+        <v>0</v>
+      </c>
+      <c r="J157" t="n">
+        <v>0</v>
+      </c>
+      <c r="K157" t="n">
+        <v>0</v>
+      </c>
+      <c r="L157" t="n">
+        <v>0</v>
+      </c>
+      <c r="M157" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Consignee</t>
+        </is>
+      </c>
+      <c r="F158" t="n">
+        <v>18</v>
+      </c>
+      <c r="G158" t="n">
+        <v>0</v>
+      </c>
+      <c r="H158" t="n">
+        <v>18</v>
+      </c>
+      <c r="I158" t="n">
+        <v>0</v>
+      </c>
+      <c r="J158" t="n">
+        <v>0</v>
+      </c>
+      <c r="K158" t="n">
+        <v>0</v>
+      </c>
+      <c r="L158" t="n">
+        <v>0</v>
+      </c>
+      <c r="M158" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F159" t="n">
+        <v>0</v>
+      </c>
+      <c r="G159" t="n">
+        <v>0</v>
+      </c>
+      <c r="H159" t="n">
+        <v>0</v>
+      </c>
+      <c r="I159" t="n">
+        <v>0</v>
+      </c>
+      <c r="J159" t="n">
+        <v>0</v>
+      </c>
+      <c r="K159" t="n">
+        <v>0</v>
+      </c>
+      <c r="L159" t="n">
+        <v>0</v>
+      </c>
+      <c r="M159" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>Shipper</t>
+        </is>
+      </c>
+      <c r="F160" t="n">
+        <v>11</v>
+      </c>
+      <c r="G160" t="n">
+        <v>0</v>
+      </c>
+      <c r="H160" t="n">
+        <v>25</v>
+      </c>
+      <c r="I160" t="n">
+        <v>0</v>
+      </c>
+      <c r="J160" t="n">
+        <v>0</v>
+      </c>
+      <c r="K160" t="n">
+        <v>0</v>
+      </c>
+      <c r="L160" t="n">
+        <v>0</v>
+      </c>
+      <c r="M160" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F161" t="n">
+        <v>0</v>
+      </c>
+      <c r="G161" t="n">
+        <v>0</v>
+      </c>
+      <c r="H161" t="n">
+        <v>1</v>
+      </c>
+      <c r="I161" t="n">
+        <v>0</v>
+      </c>
+      <c r="J161" t="n">
+        <v>0</v>
+      </c>
+      <c r="K161" t="n">
+        <v>0</v>
+      </c>
+      <c r="L161" t="n">
+        <v>0</v>
+      </c>
+      <c r="M161" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M141"/>
+  <autoFilter ref="A1:M161"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7374,7 +8354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G71"/>
+  <dimension ref="A1:G73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9444,8 +10424,66 @@
         <v>0</v>
       </c>
     </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>HAST</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>LCH27</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>28</v>
+      </c>
+      <c r="F72" t="n">
+        <v>6</v>
+      </c>
+      <c r="G72" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>HAST</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>LCH27</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>16</v>
+      </c>
+      <c r="F73" t="n">
+        <v>2</v>
+      </c>
+      <c r="G73" t="n">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G71"/>
+  <autoFilter ref="A1:G73"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
MISSING file: GATE IN BL No = yard BKG#; skip output files that are open in Excel; 08/10 HAST only
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gate-move-summary.xlsx
+++ b/docs/gate-move-summary.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Compare" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daily Summary'!$A$1:$M$161</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daily Summary'!$A$1:$M$145</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'System Compare'!$A$1:$G$73</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M161"/>
+  <dimension ref="A1:M145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7368,12 +7368,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>SMART BKK</t>
+          <t>HAST</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>BKK25</t>
+          <t>LCH27</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -7387,19 +7387,19 @@
         </is>
       </c>
       <c r="F142" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G142" t="n">
         <v>0</v>
       </c>
       <c r="H142" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="I142" t="n">
         <v>0</v>
       </c>
       <c r="J142" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="K142" t="n">
         <v>0</v>
@@ -7408,7 +7408,7 @@
         <v>0</v>
       </c>
       <c r="M142" t="n">
-        <v>5</v>
+        <v>23</v>
       </c>
     </row>
     <row r="143">
@@ -7417,12 +7417,12 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>SMART BKK</t>
+          <t>HAST</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>BKK25</t>
+          <t>LCH27</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -7436,7 +7436,7 @@
         </is>
       </c>
       <c r="F143" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G143" t="n">
         <v>0</v>
@@ -7448,7 +7448,7 @@
         <v>0</v>
       </c>
       <c r="J143" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K143" t="n">
         <v>0</v>
@@ -7457,7 +7457,7 @@
         <v>0</v>
       </c>
       <c r="M143" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="144">
@@ -7466,12 +7466,12 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>SMART BKK</t>
+          <t>HAST</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>BKK25</t>
+          <t>LCH27</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -7485,7 +7485,7 @@
         </is>
       </c>
       <c r="F144" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G144" t="n">
         <v>0</v>
@@ -7497,7 +7497,7 @@
         <v>0</v>
       </c>
       <c r="J144" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="K144" t="n">
         <v>0</v>
@@ -7506,7 +7506,7 @@
         <v>0</v>
       </c>
       <c r="M144" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="145">
@@ -7515,12 +7515,12 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>SMART BKK</t>
+          <t>HAST</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>BKK25</t>
+          <t>LCH27</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -7558,792 +7558,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146">
-      <c r="A146" s="2" t="n">
-        <v>46303</v>
-      </c>
-      <c r="B146" t="inlineStr">
-        <is>
-          <t>BC</t>
-        </is>
-      </c>
-      <c r="C146" t="inlineStr">
-        <is>
-          <t>BKK27</t>
-        </is>
-      </c>
-      <c r="D146" t="inlineStr">
-        <is>
-          <t>GATE IN</t>
-        </is>
-      </c>
-      <c r="E146" t="inlineStr">
-        <is>
-          <t>Consignee</t>
-        </is>
-      </c>
-      <c r="F146" t="n">
-        <v>70</v>
-      </c>
-      <c r="G146" t="n">
-        <v>1</v>
-      </c>
-      <c r="H146" t="n">
-        <v>29</v>
-      </c>
-      <c r="I146" t="n">
-        <v>1</v>
-      </c>
-      <c r="J146" t="n">
-        <v>4</v>
-      </c>
-      <c r="K146" t="n">
-        <v>0</v>
-      </c>
-      <c r="L146" t="n">
-        <v>0</v>
-      </c>
-      <c r="M146" t="n">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" s="2" t="n">
-        <v>46303</v>
-      </c>
-      <c r="B147" t="inlineStr">
-        <is>
-          <t>BC</t>
-        </is>
-      </c>
-      <c r="C147" t="inlineStr">
-        <is>
-          <t>BKK27</t>
-        </is>
-      </c>
-      <c r="D147" t="inlineStr">
-        <is>
-          <t>GATE IN</t>
-        </is>
-      </c>
-      <c r="E147" t="inlineStr">
-        <is>
-          <t>Agent</t>
-        </is>
-      </c>
-      <c r="F147" t="n">
-        <v>0</v>
-      </c>
-      <c r="G147" t="n">
-        <v>0</v>
-      </c>
-      <c r="H147" t="n">
-        <v>0</v>
-      </c>
-      <c r="I147" t="n">
-        <v>0</v>
-      </c>
-      <c r="J147" t="n">
-        <v>0</v>
-      </c>
-      <c r="K147" t="n">
-        <v>0</v>
-      </c>
-      <c r="L147" t="n">
-        <v>0</v>
-      </c>
-      <c r="M147" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" s="2" t="n">
-        <v>46303</v>
-      </c>
-      <c r="B148" t="inlineStr">
-        <is>
-          <t>BC</t>
-        </is>
-      </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t>BKK27</t>
-        </is>
-      </c>
-      <c r="D148" t="inlineStr">
-        <is>
-          <t>GATE OUT</t>
-        </is>
-      </c>
-      <c r="E148" t="inlineStr">
-        <is>
-          <t>Shipper</t>
-        </is>
-      </c>
-      <c r="F148" t="n">
-        <v>28</v>
-      </c>
-      <c r="G148" t="n">
-        <v>0</v>
-      </c>
-      <c r="H148" t="n">
-        <v>42</v>
-      </c>
-      <c r="I148" t="n">
-        <v>0</v>
-      </c>
-      <c r="J148" t="n">
-        <v>3</v>
-      </c>
-      <c r="K148" t="n">
-        <v>0</v>
-      </c>
-      <c r="L148" t="n">
-        <v>0</v>
-      </c>
-      <c r="M148" t="n">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" s="2" t="n">
-        <v>46303</v>
-      </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>BC</t>
-        </is>
-      </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>BKK27</t>
-        </is>
-      </c>
-      <c r="D149" t="inlineStr">
-        <is>
-          <t>GATE OUT</t>
-        </is>
-      </c>
-      <c r="E149" t="inlineStr">
-        <is>
-          <t>Agent</t>
-        </is>
-      </c>
-      <c r="F149" t="n">
-        <v>0</v>
-      </c>
-      <c r="G149" t="n">
-        <v>0</v>
-      </c>
-      <c r="H149" t="n">
-        <v>0</v>
-      </c>
-      <c r="I149" t="n">
-        <v>0</v>
-      </c>
-      <c r="J149" t="n">
-        <v>0</v>
-      </c>
-      <c r="K149" t="n">
-        <v>0</v>
-      </c>
-      <c r="L149" t="n">
-        <v>0</v>
-      </c>
-      <c r="M149" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" s="2" t="n">
-        <v>46303</v>
-      </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>HAST</t>
-        </is>
-      </c>
-      <c r="C150" t="inlineStr">
-        <is>
-          <t>LCH27</t>
-        </is>
-      </c>
-      <c r="D150" t="inlineStr">
-        <is>
-          <t>GATE IN</t>
-        </is>
-      </c>
-      <c r="E150" t="inlineStr">
-        <is>
-          <t>Consignee</t>
-        </is>
-      </c>
-      <c r="F150" t="n">
-        <v>4</v>
-      </c>
-      <c r="G150" t="n">
-        <v>0</v>
-      </c>
-      <c r="H150" t="n">
-        <v>13</v>
-      </c>
-      <c r="I150" t="n">
-        <v>0</v>
-      </c>
-      <c r="J150" t="n">
-        <v>6</v>
-      </c>
-      <c r="K150" t="n">
-        <v>0</v>
-      </c>
-      <c r="L150" t="n">
-        <v>0</v>
-      </c>
-      <c r="M150" t="n">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" s="2" t="n">
-        <v>46303</v>
-      </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>HAST</t>
-        </is>
-      </c>
-      <c r="C151" t="inlineStr">
-        <is>
-          <t>LCH27</t>
-        </is>
-      </c>
-      <c r="D151" t="inlineStr">
-        <is>
-          <t>GATE IN</t>
-        </is>
-      </c>
-      <c r="E151" t="inlineStr">
-        <is>
-          <t>Agent</t>
-        </is>
-      </c>
-      <c r="F151" t="n">
-        <v>4</v>
-      </c>
-      <c r="G151" t="n">
-        <v>0</v>
-      </c>
-      <c r="H151" t="n">
-        <v>0</v>
-      </c>
-      <c r="I151" t="n">
-        <v>0</v>
-      </c>
-      <c r="J151" t="n">
-        <v>1</v>
-      </c>
-      <c r="K151" t="n">
-        <v>0</v>
-      </c>
-      <c r="L151" t="n">
-        <v>0</v>
-      </c>
-      <c r="M151" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" s="2" t="n">
-        <v>46303</v>
-      </c>
-      <c r="B152" t="inlineStr">
-        <is>
-          <t>HAST</t>
-        </is>
-      </c>
-      <c r="C152" t="inlineStr">
-        <is>
-          <t>LCH27</t>
-        </is>
-      </c>
-      <c r="D152" t="inlineStr">
-        <is>
-          <t>GATE OUT</t>
-        </is>
-      </c>
-      <c r="E152" t="inlineStr">
-        <is>
-          <t>Shipper</t>
-        </is>
-      </c>
-      <c r="F152" t="n">
-        <v>5</v>
-      </c>
-      <c r="G152" t="n">
-        <v>0</v>
-      </c>
-      <c r="H152" t="n">
-        <v>5</v>
-      </c>
-      <c r="I152" t="n">
-        <v>0</v>
-      </c>
-      <c r="J152" t="n">
-        <v>6</v>
-      </c>
-      <c r="K152" t="n">
-        <v>0</v>
-      </c>
-      <c r="L152" t="n">
-        <v>0</v>
-      </c>
-      <c r="M152" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" s="2" t="n">
-        <v>46303</v>
-      </c>
-      <c r="B153" t="inlineStr">
-        <is>
-          <t>HAST</t>
-        </is>
-      </c>
-      <c r="C153" t="inlineStr">
-        <is>
-          <t>LCH27</t>
-        </is>
-      </c>
-      <c r="D153" t="inlineStr">
-        <is>
-          <t>GATE OUT</t>
-        </is>
-      </c>
-      <c r="E153" t="inlineStr">
-        <is>
-          <t>Agent</t>
-        </is>
-      </c>
-      <c r="F153" t="n">
-        <v>0</v>
-      </c>
-      <c r="G153" t="n">
-        <v>0</v>
-      </c>
-      <c r="H153" t="n">
-        <v>0</v>
-      </c>
-      <c r="I153" t="n">
-        <v>0</v>
-      </c>
-      <c r="J153" t="n">
-        <v>0</v>
-      </c>
-      <c r="K153" t="n">
-        <v>0</v>
-      </c>
-      <c r="L153" t="n">
-        <v>0</v>
-      </c>
-      <c r="M153" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" s="2" t="n">
-        <v>46303</v>
-      </c>
-      <c r="B154" t="inlineStr">
-        <is>
-          <t>CELLO</t>
-        </is>
-      </c>
-      <c r="C154" t="inlineStr">
-        <is>
-          <t>LCH28</t>
-        </is>
-      </c>
-      <c r="D154" t="inlineStr">
-        <is>
-          <t>GATE IN</t>
-        </is>
-      </c>
-      <c r="E154" t="inlineStr">
-        <is>
-          <t>Consignee</t>
-        </is>
-      </c>
-      <c r="F154" t="n">
-        <v>0</v>
-      </c>
-      <c r="G154" t="n">
-        <v>0</v>
-      </c>
-      <c r="H154" t="n">
-        <v>1</v>
-      </c>
-      <c r="I154" t="n">
-        <v>0</v>
-      </c>
-      <c r="J154" t="n">
-        <v>0</v>
-      </c>
-      <c r="K154" t="n">
-        <v>0</v>
-      </c>
-      <c r="L154" t="n">
-        <v>0</v>
-      </c>
-      <c r="M154" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" s="2" t="n">
-        <v>46303</v>
-      </c>
-      <c r="B155" t="inlineStr">
-        <is>
-          <t>CELLO</t>
-        </is>
-      </c>
-      <c r="C155" t="inlineStr">
-        <is>
-          <t>LCH28</t>
-        </is>
-      </c>
-      <c r="D155" t="inlineStr">
-        <is>
-          <t>GATE IN</t>
-        </is>
-      </c>
-      <c r="E155" t="inlineStr">
-        <is>
-          <t>Agent</t>
-        </is>
-      </c>
-      <c r="F155" t="n">
-        <v>0</v>
-      </c>
-      <c r="G155" t="n">
-        <v>0</v>
-      </c>
-      <c r="H155" t="n">
-        <v>0</v>
-      </c>
-      <c r="I155" t="n">
-        <v>0</v>
-      </c>
-      <c r="J155" t="n">
-        <v>0</v>
-      </c>
-      <c r="K155" t="n">
-        <v>0</v>
-      </c>
-      <c r="L155" t="n">
-        <v>0</v>
-      </c>
-      <c r="M155" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" s="2" t="n">
-        <v>46303</v>
-      </c>
-      <c r="B156" t="inlineStr">
-        <is>
-          <t>CELLO</t>
-        </is>
-      </c>
-      <c r="C156" t="inlineStr">
-        <is>
-          <t>LCH28</t>
-        </is>
-      </c>
-      <c r="D156" t="inlineStr">
-        <is>
-          <t>GATE OUT</t>
-        </is>
-      </c>
-      <c r="E156" t="inlineStr">
-        <is>
-          <t>Shipper</t>
-        </is>
-      </c>
-      <c r="F156" t="n">
-        <v>0</v>
-      </c>
-      <c r="G156" t="n">
-        <v>0</v>
-      </c>
-      <c r="H156" t="n">
-        <v>0</v>
-      </c>
-      <c r="I156" t="n">
-        <v>0</v>
-      </c>
-      <c r="J156" t="n">
-        <v>0</v>
-      </c>
-      <c r="K156" t="n">
-        <v>0</v>
-      </c>
-      <c r="L156" t="n">
-        <v>0</v>
-      </c>
-      <c r="M156" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" s="2" t="n">
-        <v>46303</v>
-      </c>
-      <c r="B157" t="inlineStr">
-        <is>
-          <t>CELLO</t>
-        </is>
-      </c>
-      <c r="C157" t="inlineStr">
-        <is>
-          <t>LCH28</t>
-        </is>
-      </c>
-      <c r="D157" t="inlineStr">
-        <is>
-          <t>GATE OUT</t>
-        </is>
-      </c>
-      <c r="E157" t="inlineStr">
-        <is>
-          <t>Agent</t>
-        </is>
-      </c>
-      <c r="F157" t="n">
-        <v>0</v>
-      </c>
-      <c r="G157" t="n">
-        <v>0</v>
-      </c>
-      <c r="H157" t="n">
-        <v>0</v>
-      </c>
-      <c r="I157" t="n">
-        <v>0</v>
-      </c>
-      <c r="J157" t="n">
-        <v>0</v>
-      </c>
-      <c r="K157" t="n">
-        <v>0</v>
-      </c>
-      <c r="L157" t="n">
-        <v>0</v>
-      </c>
-      <c r="M157" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" s="2" t="n">
-        <v>46303</v>
-      </c>
-      <c r="B158" t="inlineStr">
-        <is>
-          <t>PW</t>
-        </is>
-      </c>
-      <c r="C158" t="inlineStr">
-        <is>
-          <t>LCHY5</t>
-        </is>
-      </c>
-      <c r="D158" t="inlineStr">
-        <is>
-          <t>GATE IN</t>
-        </is>
-      </c>
-      <c r="E158" t="inlineStr">
-        <is>
-          <t>Consignee</t>
-        </is>
-      </c>
-      <c r="F158" t="n">
-        <v>18</v>
-      </c>
-      <c r="G158" t="n">
-        <v>0</v>
-      </c>
-      <c r="H158" t="n">
-        <v>18</v>
-      </c>
-      <c r="I158" t="n">
-        <v>0</v>
-      </c>
-      <c r="J158" t="n">
-        <v>0</v>
-      </c>
-      <c r="K158" t="n">
-        <v>0</v>
-      </c>
-      <c r="L158" t="n">
-        <v>0</v>
-      </c>
-      <c r="M158" t="n">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" s="2" t="n">
-        <v>46303</v>
-      </c>
-      <c r="B159" t="inlineStr">
-        <is>
-          <t>PW</t>
-        </is>
-      </c>
-      <c r="C159" t="inlineStr">
-        <is>
-          <t>LCHY5</t>
-        </is>
-      </c>
-      <c r="D159" t="inlineStr">
-        <is>
-          <t>GATE IN</t>
-        </is>
-      </c>
-      <c r="E159" t="inlineStr">
-        <is>
-          <t>Agent</t>
-        </is>
-      </c>
-      <c r="F159" t="n">
-        <v>0</v>
-      </c>
-      <c r="G159" t="n">
-        <v>0</v>
-      </c>
-      <c r="H159" t="n">
-        <v>0</v>
-      </c>
-      <c r="I159" t="n">
-        <v>0</v>
-      </c>
-      <c r="J159" t="n">
-        <v>0</v>
-      </c>
-      <c r="K159" t="n">
-        <v>0</v>
-      </c>
-      <c r="L159" t="n">
-        <v>0</v>
-      </c>
-      <c r="M159" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" s="2" t="n">
-        <v>46303</v>
-      </c>
-      <c r="B160" t="inlineStr">
-        <is>
-          <t>PW</t>
-        </is>
-      </c>
-      <c r="C160" t="inlineStr">
-        <is>
-          <t>LCHY5</t>
-        </is>
-      </c>
-      <c r="D160" t="inlineStr">
-        <is>
-          <t>GATE OUT</t>
-        </is>
-      </c>
-      <c r="E160" t="inlineStr">
-        <is>
-          <t>Shipper</t>
-        </is>
-      </c>
-      <c r="F160" t="n">
-        <v>11</v>
-      </c>
-      <c r="G160" t="n">
-        <v>0</v>
-      </c>
-      <c r="H160" t="n">
-        <v>25</v>
-      </c>
-      <c r="I160" t="n">
-        <v>0</v>
-      </c>
-      <c r="J160" t="n">
-        <v>0</v>
-      </c>
-      <c r="K160" t="n">
-        <v>0</v>
-      </c>
-      <c r="L160" t="n">
-        <v>0</v>
-      </c>
-      <c r="M160" t="n">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" s="2" t="n">
-        <v>46303</v>
-      </c>
-      <c r="B161" t="inlineStr">
-        <is>
-          <t>PW</t>
-        </is>
-      </c>
-      <c r="C161" t="inlineStr">
-        <is>
-          <t>LCHY5</t>
-        </is>
-      </c>
-      <c r="D161" t="inlineStr">
-        <is>
-          <t>GATE OUT</t>
-        </is>
-      </c>
-      <c r="E161" t="inlineStr">
-        <is>
-          <t>Agent</t>
-        </is>
-      </c>
-      <c r="F161" t="n">
-        <v>0</v>
-      </c>
-      <c r="G161" t="n">
-        <v>0</v>
-      </c>
-      <c r="H161" t="n">
-        <v>1</v>
-      </c>
-      <c r="I161" t="n">
-        <v>0</v>
-      </c>
-      <c r="J161" t="n">
-        <v>0</v>
-      </c>
-      <c r="K161" t="n">
-        <v>0</v>
-      </c>
-      <c r="L161" t="n">
-        <v>0</v>
-      </c>
-      <c r="M161" t="n">
-        <v>1</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:M161"/>
+  <autoFilter ref="A1:M145"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Database: re-running replaces only the yards in the run; 08/10 PW
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gate-move-summary.xlsx
+++ b/docs/gate-move-summary.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Compare" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daily Summary'!$A$1:$M$145</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'System Compare'!$A$1:$G$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daily Summary'!$A$1:$M$149</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'System Compare'!$A$1:$G$75</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M145"/>
+  <dimension ref="A1:M149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7558,8 +7558,204 @@
         <v>0</v>
       </c>
     </row>
+    <row r="146">
+      <c r="A146" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Consignee</t>
+        </is>
+      </c>
+      <c r="F146" t="n">
+        <v>18</v>
+      </c>
+      <c r="G146" t="n">
+        <v>0</v>
+      </c>
+      <c r="H146" t="n">
+        <v>18</v>
+      </c>
+      <c r="I146" t="n">
+        <v>0</v>
+      </c>
+      <c r="J146" t="n">
+        <v>0</v>
+      </c>
+      <c r="K146" t="n">
+        <v>0</v>
+      </c>
+      <c r="L146" t="n">
+        <v>0</v>
+      </c>
+      <c r="M146" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F147" t="n">
+        <v>0</v>
+      </c>
+      <c r="G147" t="n">
+        <v>0</v>
+      </c>
+      <c r="H147" t="n">
+        <v>0</v>
+      </c>
+      <c r="I147" t="n">
+        <v>0</v>
+      </c>
+      <c r="J147" t="n">
+        <v>0</v>
+      </c>
+      <c r="K147" t="n">
+        <v>0</v>
+      </c>
+      <c r="L147" t="n">
+        <v>0</v>
+      </c>
+      <c r="M147" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Shipper</t>
+        </is>
+      </c>
+      <c r="F148" t="n">
+        <v>11</v>
+      </c>
+      <c r="G148" t="n">
+        <v>0</v>
+      </c>
+      <c r="H148" t="n">
+        <v>25</v>
+      </c>
+      <c r="I148" t="n">
+        <v>0</v>
+      </c>
+      <c r="J148" t="n">
+        <v>0</v>
+      </c>
+      <c r="K148" t="n">
+        <v>0</v>
+      </c>
+      <c r="L148" t="n">
+        <v>0</v>
+      </c>
+      <c r="M148" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F149" t="n">
+        <v>0</v>
+      </c>
+      <c r="G149" t="n">
+        <v>0</v>
+      </c>
+      <c r="H149" t="n">
+        <v>1</v>
+      </c>
+      <c r="I149" t="n">
+        <v>0</v>
+      </c>
+      <c r="J149" t="n">
+        <v>0</v>
+      </c>
+      <c r="K149" t="n">
+        <v>0</v>
+      </c>
+      <c r="L149" t="n">
+        <v>0</v>
+      </c>
+      <c r="M149" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M145"/>
+  <autoFilter ref="A1:M149"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7570,7 +7766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G73"/>
+  <dimension ref="A1:G75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9698,8 +9894,66 @@
         <v>14</v>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>36</v>
+      </c>
+      <c r="F74" t="n">
+        <v>35</v>
+      </c>
+      <c r="G74" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>37</v>
+      </c>
+      <c r="F75" t="n">
+        <v>37</v>
+      </c>
+      <c r="G75" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G73"/>
+  <autoFilter ref="A1:G75"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 08/10/2026 data (all yards, 10-8-GAF)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gate-move-summary.xlsx
+++ b/docs/gate-move-summary.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Compare" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daily Summary'!$A$1:$M$149</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'System Compare'!$A$1:$G$75</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daily Summary'!$A$1:$M$161</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'System Compare'!$A$1:$G$81</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M149"/>
+  <dimension ref="A1:M161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7368,12 +7368,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>HAST</t>
+          <t>SMART BKK</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>LCH27</t>
+          <t>BKK25</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -7387,19 +7387,19 @@
         </is>
       </c>
       <c r="F142" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G142" t="n">
         <v>0</v>
       </c>
       <c r="H142" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="I142" t="n">
         <v>0</v>
       </c>
       <c r="J142" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K142" t="n">
         <v>0</v>
@@ -7408,7 +7408,7 @@
         <v>0</v>
       </c>
       <c r="M142" t="n">
-        <v>23</v>
+        <v>5</v>
       </c>
     </row>
     <row r="143">
@@ -7417,12 +7417,12 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>HAST</t>
+          <t>SMART BKK</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>LCH27</t>
+          <t>BKK25</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -7436,7 +7436,7 @@
         </is>
       </c>
       <c r="F143" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G143" t="n">
         <v>0</v>
@@ -7448,7 +7448,7 @@
         <v>0</v>
       </c>
       <c r="J143" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K143" t="n">
         <v>0</v>
@@ -7457,7 +7457,7 @@
         <v>0</v>
       </c>
       <c r="M143" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="144">
@@ -7466,12 +7466,12 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>HAST</t>
+          <t>SMART BKK</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>LCH27</t>
+          <t>BKK25</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -7485,7 +7485,7 @@
         </is>
       </c>
       <c r="F144" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G144" t="n">
         <v>0</v>
@@ -7497,7 +7497,7 @@
         <v>0</v>
       </c>
       <c r="J144" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K144" t="n">
         <v>0</v>
@@ -7506,7 +7506,7 @@
         <v>0</v>
       </c>
       <c r="M144" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
     </row>
     <row r="145">
@@ -7515,12 +7515,12 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>HAST</t>
+          <t>SMART BKK</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>LCH27</t>
+          <t>BKK25</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -7564,12 +7564,12 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>PW</t>
+          <t>BC</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>LCHY5</t>
+          <t>BKK27</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -7583,19 +7583,19 @@
         </is>
       </c>
       <c r="F146" t="n">
-        <v>18</v>
+        <v>70</v>
       </c>
       <c r="G146" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H146" t="n">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="I146" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J146" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K146" t="n">
         <v>0</v>
@@ -7604,7 +7604,7 @@
         <v>0</v>
       </c>
       <c r="M146" t="n">
-        <v>36</v>
+        <v>105</v>
       </c>
     </row>
     <row r="147">
@@ -7613,12 +7613,12 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>PW</t>
+          <t>BC</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>LCHY5</t>
+          <t>BKK27</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -7662,12 +7662,12 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>PW</t>
+          <t>BC</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>LCHY5</t>
+          <t>BKK27</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -7681,19 +7681,19 @@
         </is>
       </c>
       <c r="F148" t="n">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="G148" t="n">
         <v>0</v>
       </c>
       <c r="H148" t="n">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="I148" t="n">
         <v>0</v>
       </c>
       <c r="J148" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K148" t="n">
         <v>0</v>
@@ -7702,7 +7702,7 @@
         <v>0</v>
       </c>
       <c r="M148" t="n">
-        <v>36</v>
+        <v>76</v>
       </c>
     </row>
     <row r="149">
@@ -7711,51 +7711,639 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>BKK27</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F149" t="n">
+        <v>0</v>
+      </c>
+      <c r="G149" t="n">
+        <v>0</v>
+      </c>
+      <c r="H149" t="n">
+        <v>0</v>
+      </c>
+      <c r="I149" t="n">
+        <v>0</v>
+      </c>
+      <c r="J149" t="n">
+        <v>0</v>
+      </c>
+      <c r="K149" t="n">
+        <v>0</v>
+      </c>
+      <c r="L149" t="n">
+        <v>0</v>
+      </c>
+      <c r="M149" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>HAST</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>LCH27</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>Consignee</t>
+        </is>
+      </c>
+      <c r="F150" t="n">
+        <v>4</v>
+      </c>
+      <c r="G150" t="n">
+        <v>0</v>
+      </c>
+      <c r="H150" t="n">
+        <v>13</v>
+      </c>
+      <c r="I150" t="n">
+        <v>0</v>
+      </c>
+      <c r="J150" t="n">
+        <v>6</v>
+      </c>
+      <c r="K150" t="n">
+        <v>0</v>
+      </c>
+      <c r="L150" t="n">
+        <v>0</v>
+      </c>
+      <c r="M150" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>HAST</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>LCH27</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F151" t="n">
+        <v>4</v>
+      </c>
+      <c r="G151" t="n">
+        <v>0</v>
+      </c>
+      <c r="H151" t="n">
+        <v>0</v>
+      </c>
+      <c r="I151" t="n">
+        <v>0</v>
+      </c>
+      <c r="J151" t="n">
+        <v>1</v>
+      </c>
+      <c r="K151" t="n">
+        <v>0</v>
+      </c>
+      <c r="L151" t="n">
+        <v>0</v>
+      </c>
+      <c r="M151" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>HAST</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>LCH27</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Shipper</t>
+        </is>
+      </c>
+      <c r="F152" t="n">
+        <v>5</v>
+      </c>
+      <c r="G152" t="n">
+        <v>0</v>
+      </c>
+      <c r="H152" t="n">
+        <v>5</v>
+      </c>
+      <c r="I152" t="n">
+        <v>0</v>
+      </c>
+      <c r="J152" t="n">
+        <v>6</v>
+      </c>
+      <c r="K152" t="n">
+        <v>0</v>
+      </c>
+      <c r="L152" t="n">
+        <v>0</v>
+      </c>
+      <c r="M152" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>HAST</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>LCH27</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F153" t="n">
+        <v>0</v>
+      </c>
+      <c r="G153" t="n">
+        <v>0</v>
+      </c>
+      <c r="H153" t="n">
+        <v>0</v>
+      </c>
+      <c r="I153" t="n">
+        <v>0</v>
+      </c>
+      <c r="J153" t="n">
+        <v>0</v>
+      </c>
+      <c r="K153" t="n">
+        <v>0</v>
+      </c>
+      <c r="L153" t="n">
+        <v>0</v>
+      </c>
+      <c r="M153" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>LCH28</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Consignee</t>
+        </is>
+      </c>
+      <c r="F154" t="n">
+        <v>0</v>
+      </c>
+      <c r="G154" t="n">
+        <v>0</v>
+      </c>
+      <c r="H154" t="n">
+        <v>1</v>
+      </c>
+      <c r="I154" t="n">
+        <v>0</v>
+      </c>
+      <c r="J154" t="n">
+        <v>0</v>
+      </c>
+      <c r="K154" t="n">
+        <v>0</v>
+      </c>
+      <c r="L154" t="n">
+        <v>0</v>
+      </c>
+      <c r="M154" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>LCH28</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F155" t="n">
+        <v>0</v>
+      </c>
+      <c r="G155" t="n">
+        <v>0</v>
+      </c>
+      <c r="H155" t="n">
+        <v>0</v>
+      </c>
+      <c r="I155" t="n">
+        <v>0</v>
+      </c>
+      <c r="J155" t="n">
+        <v>0</v>
+      </c>
+      <c r="K155" t="n">
+        <v>0</v>
+      </c>
+      <c r="L155" t="n">
+        <v>0</v>
+      </c>
+      <c r="M155" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>LCH28</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Shipper</t>
+        </is>
+      </c>
+      <c r="F156" t="n">
+        <v>0</v>
+      </c>
+      <c r="G156" t="n">
+        <v>0</v>
+      </c>
+      <c r="H156" t="n">
+        <v>0</v>
+      </c>
+      <c r="I156" t="n">
+        <v>0</v>
+      </c>
+      <c r="J156" t="n">
+        <v>0</v>
+      </c>
+      <c r="K156" t="n">
+        <v>0</v>
+      </c>
+      <c r="L156" t="n">
+        <v>0</v>
+      </c>
+      <c r="M156" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>LCH28</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F157" t="n">
+        <v>0</v>
+      </c>
+      <c r="G157" t="n">
+        <v>0</v>
+      </c>
+      <c r="H157" t="n">
+        <v>0</v>
+      </c>
+      <c r="I157" t="n">
+        <v>0</v>
+      </c>
+      <c r="J157" t="n">
+        <v>0</v>
+      </c>
+      <c r="K157" t="n">
+        <v>0</v>
+      </c>
+      <c r="L157" t="n">
+        <v>0</v>
+      </c>
+      <c r="M157" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
           <t>PW</t>
         </is>
       </c>
-      <c r="C149" t="inlineStr">
+      <c r="C158" t="inlineStr">
         <is>
           <t>LCHY5</t>
         </is>
       </c>
-      <c r="D149" t="inlineStr">
-        <is>
-          <t>GATE OUT</t>
-        </is>
-      </c>
-      <c r="E149" t="inlineStr">
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Consignee</t>
+        </is>
+      </c>
+      <c r="F158" t="n">
+        <v>18</v>
+      </c>
+      <c r="G158" t="n">
+        <v>0</v>
+      </c>
+      <c r="H158" t="n">
+        <v>18</v>
+      </c>
+      <c r="I158" t="n">
+        <v>0</v>
+      </c>
+      <c r="J158" t="n">
+        <v>0</v>
+      </c>
+      <c r="K158" t="n">
+        <v>0</v>
+      </c>
+      <c r="L158" t="n">
+        <v>0</v>
+      </c>
+      <c r="M158" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
         <is>
           <t>Agent</t>
         </is>
       </c>
-      <c r="F149" t="n">
-        <v>0</v>
-      </c>
-      <c r="G149" t="n">
-        <v>0</v>
-      </c>
-      <c r="H149" t="n">
+      <c r="F159" t="n">
+        <v>0</v>
+      </c>
+      <c r="G159" t="n">
+        <v>0</v>
+      </c>
+      <c r="H159" t="n">
+        <v>0</v>
+      </c>
+      <c r="I159" t="n">
+        <v>0</v>
+      </c>
+      <c r="J159" t="n">
+        <v>0</v>
+      </c>
+      <c r="K159" t="n">
+        <v>0</v>
+      </c>
+      <c r="L159" t="n">
+        <v>0</v>
+      </c>
+      <c r="M159" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>Shipper</t>
+        </is>
+      </c>
+      <c r="F160" t="n">
+        <v>11</v>
+      </c>
+      <c r="G160" t="n">
+        <v>0</v>
+      </c>
+      <c r="H160" t="n">
+        <v>25</v>
+      </c>
+      <c r="I160" t="n">
+        <v>0</v>
+      </c>
+      <c r="J160" t="n">
+        <v>0</v>
+      </c>
+      <c r="K160" t="n">
+        <v>0</v>
+      </c>
+      <c r="L160" t="n">
+        <v>0</v>
+      </c>
+      <c r="M160" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F161" t="n">
+        <v>0</v>
+      </c>
+      <c r="G161" t="n">
+        <v>0</v>
+      </c>
+      <c r="H161" t="n">
         <v>1</v>
       </c>
-      <c r="I149" t="n">
-        <v>0</v>
-      </c>
-      <c r="J149" t="n">
-        <v>0</v>
-      </c>
-      <c r="K149" t="n">
-        <v>0</v>
-      </c>
-      <c r="L149" t="n">
-        <v>0</v>
-      </c>
-      <c r="M149" t="n">
+      <c r="I161" t="n">
+        <v>0</v>
+      </c>
+      <c r="J161" t="n">
+        <v>0</v>
+      </c>
+      <c r="K161" t="n">
+        <v>0</v>
+      </c>
+      <c r="L161" t="n">
+        <v>0</v>
+      </c>
+      <c r="M161" t="n">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M149"/>
+  <autoFilter ref="A1:M161"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7766,7 +8354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G75"/>
+  <dimension ref="A1:G81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9842,12 +10430,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>HAST</t>
+          <t>SMART BKK</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>LCH27</t>
+          <t>BKK25</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -9856,13 +10444,13 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="F72" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G72" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73">
@@ -9871,12 +10459,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>HAST</t>
+          <t>SMART BKK</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>LCH27</t>
+          <t>BKK25</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -9885,13 +10473,13 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="F73" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="G73" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74">
@@ -9900,12 +10488,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>PW</t>
+          <t>BC</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>LCHY5</t>
+          <t>BKK27</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -9914,13 +10502,13 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>36</v>
+        <v>105</v>
       </c>
       <c r="F74" t="n">
-        <v>35</v>
+        <v>105</v>
       </c>
       <c r="G74" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75">
@@ -9929,31 +10517,205 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>BKK27</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>76</v>
+      </c>
+      <c r="F75" t="n">
+        <v>76</v>
+      </c>
+      <c r="G75" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>HAST</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>LCH27</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>28</v>
+      </c>
+      <c r="F76" t="n">
+        <v>28</v>
+      </c>
+      <c r="G76" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>HAST</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>LCH27</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>16</v>
+      </c>
+      <c r="F77" t="n">
+        <v>16</v>
+      </c>
+      <c r="G77" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>LCH28</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>1</v>
+      </c>
+      <c r="F78" t="n">
+        <v>1</v>
+      </c>
+      <c r="G78" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>LCH28</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>0</v>
+      </c>
+      <c r="F79" t="n">
+        <v>0</v>
+      </c>
+      <c r="G79" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
           <t>PW</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
+      <c r="C80" t="inlineStr">
         <is>
           <t>LCHY5</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>GATE OUT</t>
-        </is>
-      </c>
-      <c r="E75" t="n">
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>36</v>
+      </c>
+      <c r="F80" t="n">
+        <v>36</v>
+      </c>
+      <c r="G80" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
         <v>37</v>
       </c>
-      <c r="F75" t="n">
+      <c r="F81" t="n">
         <v>37</v>
       </c>
-      <c r="G75" t="n">
+      <c r="G81" t="n">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G75"/>
+  <autoFilter ref="A1:G81"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Any .xls in a given source folder can be the system export; 09/10 PW
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gate-move-summary.xlsx
+++ b/docs/gate-move-summary.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Compare" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daily Summary'!$A$1:$M$161</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'System Compare'!$A$1:$G$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daily Summary'!$A$1:$M$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'System Compare'!$A$1:$G$83</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M161"/>
+  <dimension ref="A1:M165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8342,8 +8342,204 @@
         <v>1</v>
       </c>
     </row>
+    <row r="162">
+      <c r="A162" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>Consignee</t>
+        </is>
+      </c>
+      <c r="F162" t="n">
+        <v>60</v>
+      </c>
+      <c r="G162" t="n">
+        <v>0</v>
+      </c>
+      <c r="H162" t="n">
+        <v>18</v>
+      </c>
+      <c r="I162" t="n">
+        <v>0</v>
+      </c>
+      <c r="J162" t="n">
+        <v>0</v>
+      </c>
+      <c r="K162" t="n">
+        <v>0</v>
+      </c>
+      <c r="L162" t="n">
+        <v>0</v>
+      </c>
+      <c r="M162" t="n">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F163" t="n">
+        <v>0</v>
+      </c>
+      <c r="G163" t="n">
+        <v>0</v>
+      </c>
+      <c r="H163" t="n">
+        <v>0</v>
+      </c>
+      <c r="I163" t="n">
+        <v>0</v>
+      </c>
+      <c r="J163" t="n">
+        <v>0</v>
+      </c>
+      <c r="K163" t="n">
+        <v>0</v>
+      </c>
+      <c r="L163" t="n">
+        <v>0</v>
+      </c>
+      <c r="M163" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>Shipper</t>
+        </is>
+      </c>
+      <c r="F164" t="n">
+        <v>26</v>
+      </c>
+      <c r="G164" t="n">
+        <v>0</v>
+      </c>
+      <c r="H164" t="n">
+        <v>18</v>
+      </c>
+      <c r="I164" t="n">
+        <v>0</v>
+      </c>
+      <c r="J164" t="n">
+        <v>0</v>
+      </c>
+      <c r="K164" t="n">
+        <v>0</v>
+      </c>
+      <c r="L164" t="n">
+        <v>0</v>
+      </c>
+      <c r="M164" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F165" t="n">
+        <v>0</v>
+      </c>
+      <c r="G165" t="n">
+        <v>0</v>
+      </c>
+      <c r="H165" t="n">
+        <v>0</v>
+      </c>
+      <c r="I165" t="n">
+        <v>0</v>
+      </c>
+      <c r="J165" t="n">
+        <v>0</v>
+      </c>
+      <c r="K165" t="n">
+        <v>0</v>
+      </c>
+      <c r="L165" t="n">
+        <v>0</v>
+      </c>
+      <c r="M165" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M161"/>
+  <autoFilter ref="A1:M165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8354,7 +8550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G81"/>
+  <dimension ref="A1:G83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10714,8 +10910,66 @@
         <v>0</v>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>78</v>
+      </c>
+      <c r="F82" t="n">
+        <v>66</v>
+      </c>
+      <c r="G82" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>44</v>
+      </c>
+      <c r="F83" t="n">
+        <v>39</v>
+      </c>
+      <c r="G83" t="n">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G81"/>
+  <autoFilter ref="A1:G83"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Pick job no. out of longer GATE OUT notes; add 09/10/2026 (all yards)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gate-move-summary.xlsx
+++ b/docs/gate-move-summary.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Compare" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daily Summary'!$A$1:$M$165</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'System Compare'!$A$1:$G$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daily Summary'!$A$1:$M$181</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'System Compare'!$A$1:$G$91</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M165"/>
+  <dimension ref="A1:M181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8348,12 +8348,12 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>PW</t>
+          <t>SMART BKK</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>LCHY5</t>
+          <t>BKK25</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -8367,13 +8367,13 @@
         </is>
       </c>
       <c r="F162" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="G162" t="n">
         <v>0</v>
       </c>
       <c r="H162" t="n">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="I162" t="n">
         <v>0</v>
@@ -8388,7 +8388,7 @@
         <v>0</v>
       </c>
       <c r="M162" t="n">
-        <v>78</v>
+        <v>3</v>
       </c>
     </row>
     <row r="163">
@@ -8397,12 +8397,12 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>PW</t>
+          <t>SMART BKK</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>LCHY5</t>
+          <t>BKK25</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -8446,12 +8446,12 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>PW</t>
+          <t>SMART BKK</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>LCHY5</t>
+          <t>BKK25</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -8465,13 +8465,13 @@
         </is>
       </c>
       <c r="F164" t="n">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="G164" t="n">
         <v>0</v>
       </c>
       <c r="H164" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="I164" t="n">
         <v>0</v>
@@ -8486,7 +8486,7 @@
         <v>0</v>
       </c>
       <c r="M164" t="n">
-        <v>44</v>
+        <v>13</v>
       </c>
     </row>
     <row r="165">
@@ -8495,51 +8495,835 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
+          <t>SMART BKK</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>BKK25</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F165" t="n">
+        <v>0</v>
+      </c>
+      <c r="G165" t="n">
+        <v>0</v>
+      </c>
+      <c r="H165" t="n">
+        <v>0</v>
+      </c>
+      <c r="I165" t="n">
+        <v>0</v>
+      </c>
+      <c r="J165" t="n">
+        <v>0</v>
+      </c>
+      <c r="K165" t="n">
+        <v>0</v>
+      </c>
+      <c r="L165" t="n">
+        <v>0</v>
+      </c>
+      <c r="M165" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>BKK27</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>Consignee</t>
+        </is>
+      </c>
+      <c r="F166" t="n">
+        <v>54</v>
+      </c>
+      <c r="G166" t="n">
+        <v>0</v>
+      </c>
+      <c r="H166" t="n">
+        <v>45</v>
+      </c>
+      <c r="I166" t="n">
+        <v>3</v>
+      </c>
+      <c r="J166" t="n">
+        <v>1</v>
+      </c>
+      <c r="K166" t="n">
+        <v>0</v>
+      </c>
+      <c r="L166" t="n">
+        <v>0</v>
+      </c>
+      <c r="M166" t="n">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>BKK27</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F167" t="n">
+        <v>8</v>
+      </c>
+      <c r="G167" t="n">
+        <v>0</v>
+      </c>
+      <c r="H167" t="n">
+        <v>0</v>
+      </c>
+      <c r="I167" t="n">
+        <v>0</v>
+      </c>
+      <c r="J167" t="n">
+        <v>0</v>
+      </c>
+      <c r="K167" t="n">
+        <v>0</v>
+      </c>
+      <c r="L167" t="n">
+        <v>0</v>
+      </c>
+      <c r="M167" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>BKK27</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>Shipper</t>
+        </is>
+      </c>
+      <c r="F168" t="n">
+        <v>25</v>
+      </c>
+      <c r="G168" t="n">
+        <v>0</v>
+      </c>
+      <c r="H168" t="n">
+        <v>19</v>
+      </c>
+      <c r="I168" t="n">
+        <v>1</v>
+      </c>
+      <c r="J168" t="n">
+        <v>0</v>
+      </c>
+      <c r="K168" t="n">
+        <v>0</v>
+      </c>
+      <c r="L168" t="n">
+        <v>0</v>
+      </c>
+      <c r="M168" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>BKK27</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F169" t="n">
+        <v>0</v>
+      </c>
+      <c r="G169" t="n">
+        <v>0</v>
+      </c>
+      <c r="H169" t="n">
+        <v>0</v>
+      </c>
+      <c r="I169" t="n">
+        <v>0</v>
+      </c>
+      <c r="J169" t="n">
+        <v>1</v>
+      </c>
+      <c r="K169" t="n">
+        <v>0</v>
+      </c>
+      <c r="L169" t="n">
+        <v>0</v>
+      </c>
+      <c r="M169" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>HAST</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>LCH27</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>Consignee</t>
+        </is>
+      </c>
+      <c r="F170" t="n">
+        <v>8</v>
+      </c>
+      <c r="G170" t="n">
+        <v>0</v>
+      </c>
+      <c r="H170" t="n">
+        <v>14</v>
+      </c>
+      <c r="I170" t="n">
+        <v>0</v>
+      </c>
+      <c r="J170" t="n">
+        <v>7</v>
+      </c>
+      <c r="K170" t="n">
+        <v>0</v>
+      </c>
+      <c r="L170" t="n">
+        <v>0</v>
+      </c>
+      <c r="M170" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>HAST</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>LCH27</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F171" t="n">
+        <v>6</v>
+      </c>
+      <c r="G171" t="n">
+        <v>0</v>
+      </c>
+      <c r="H171" t="n">
+        <v>1</v>
+      </c>
+      <c r="I171" t="n">
+        <v>0</v>
+      </c>
+      <c r="J171" t="n">
+        <v>1</v>
+      </c>
+      <c r="K171" t="n">
+        <v>0</v>
+      </c>
+      <c r="L171" t="n">
+        <v>0</v>
+      </c>
+      <c r="M171" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>HAST</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>LCH27</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>Shipper</t>
+        </is>
+      </c>
+      <c r="F172" t="n">
+        <v>5</v>
+      </c>
+      <c r="G172" t="n">
+        <v>0</v>
+      </c>
+      <c r="H172" t="n">
+        <v>17</v>
+      </c>
+      <c r="I172" t="n">
+        <v>0</v>
+      </c>
+      <c r="J172" t="n">
+        <v>4</v>
+      </c>
+      <c r="K172" t="n">
+        <v>0</v>
+      </c>
+      <c r="L172" t="n">
+        <v>0</v>
+      </c>
+      <c r="M172" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>HAST</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>LCH27</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F173" t="n">
+        <v>2</v>
+      </c>
+      <c r="G173" t="n">
+        <v>0</v>
+      </c>
+      <c r="H173" t="n">
+        <v>2</v>
+      </c>
+      <c r="I173" t="n">
+        <v>0</v>
+      </c>
+      <c r="J173" t="n">
+        <v>0</v>
+      </c>
+      <c r="K173" t="n">
+        <v>0</v>
+      </c>
+      <c r="L173" t="n">
+        <v>0</v>
+      </c>
+      <c r="M173" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>LCH28</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>Consignee</t>
+        </is>
+      </c>
+      <c r="F174" t="n">
+        <v>0</v>
+      </c>
+      <c r="G174" t="n">
+        <v>0</v>
+      </c>
+      <c r="H174" t="n">
+        <v>3</v>
+      </c>
+      <c r="I174" t="n">
+        <v>0</v>
+      </c>
+      <c r="J174" t="n">
+        <v>0</v>
+      </c>
+      <c r="K174" t="n">
+        <v>0</v>
+      </c>
+      <c r="L174" t="n">
+        <v>0</v>
+      </c>
+      <c r="M174" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>LCH28</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F175" t="n">
+        <v>0</v>
+      </c>
+      <c r="G175" t="n">
+        <v>0</v>
+      </c>
+      <c r="H175" t="n">
+        <v>0</v>
+      </c>
+      <c r="I175" t="n">
+        <v>0</v>
+      </c>
+      <c r="J175" t="n">
+        <v>0</v>
+      </c>
+      <c r="K175" t="n">
+        <v>0</v>
+      </c>
+      <c r="L175" t="n">
+        <v>0</v>
+      </c>
+      <c r="M175" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>LCH28</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>Shipper</t>
+        </is>
+      </c>
+      <c r="F176" t="n">
+        <v>0</v>
+      </c>
+      <c r="G176" t="n">
+        <v>0</v>
+      </c>
+      <c r="H176" t="n">
+        <v>1</v>
+      </c>
+      <c r="I176" t="n">
+        <v>0</v>
+      </c>
+      <c r="J176" t="n">
+        <v>0</v>
+      </c>
+      <c r="K176" t="n">
+        <v>0</v>
+      </c>
+      <c r="L176" t="n">
+        <v>0</v>
+      </c>
+      <c r="M176" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>LCH28</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F177" t="n">
+        <v>1</v>
+      </c>
+      <c r="G177" t="n">
+        <v>0</v>
+      </c>
+      <c r="H177" t="n">
+        <v>0</v>
+      </c>
+      <c r="I177" t="n">
+        <v>0</v>
+      </c>
+      <c r="J177" t="n">
+        <v>0</v>
+      </c>
+      <c r="K177" t="n">
+        <v>0</v>
+      </c>
+      <c r="L177" t="n">
+        <v>0</v>
+      </c>
+      <c r="M177" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
           <t>PW</t>
         </is>
       </c>
-      <c r="C165" t="inlineStr">
+      <c r="C178" t="inlineStr">
         <is>
           <t>LCHY5</t>
         </is>
       </c>
-      <c r="D165" t="inlineStr">
-        <is>
-          <t>GATE OUT</t>
-        </is>
-      </c>
-      <c r="E165" t="inlineStr">
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>Consignee</t>
+        </is>
+      </c>
+      <c r="F178" t="n">
+        <v>60</v>
+      </c>
+      <c r="G178" t="n">
+        <v>0</v>
+      </c>
+      <c r="H178" t="n">
+        <v>18</v>
+      </c>
+      <c r="I178" t="n">
+        <v>0</v>
+      </c>
+      <c r="J178" t="n">
+        <v>0</v>
+      </c>
+      <c r="K178" t="n">
+        <v>0</v>
+      </c>
+      <c r="L178" t="n">
+        <v>0</v>
+      </c>
+      <c r="M178" t="n">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
         <is>
           <t>Agent</t>
         </is>
       </c>
-      <c r="F165" t="n">
-        <v>0</v>
-      </c>
-      <c r="G165" t="n">
-        <v>0</v>
-      </c>
-      <c r="H165" t="n">
-        <v>0</v>
-      </c>
-      <c r="I165" t="n">
-        <v>0</v>
-      </c>
-      <c r="J165" t="n">
-        <v>0</v>
-      </c>
-      <c r="K165" t="n">
-        <v>0</v>
-      </c>
-      <c r="L165" t="n">
-        <v>0</v>
-      </c>
-      <c r="M165" t="n">
+      <c r="F179" t="n">
+        <v>0</v>
+      </c>
+      <c r="G179" t="n">
+        <v>0</v>
+      </c>
+      <c r="H179" t="n">
+        <v>0</v>
+      </c>
+      <c r="I179" t="n">
+        <v>0</v>
+      </c>
+      <c r="J179" t="n">
+        <v>0</v>
+      </c>
+      <c r="K179" t="n">
+        <v>0</v>
+      </c>
+      <c r="L179" t="n">
+        <v>0</v>
+      </c>
+      <c r="M179" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>Shipper</t>
+        </is>
+      </c>
+      <c r="F180" t="n">
+        <v>26</v>
+      </c>
+      <c r="G180" t="n">
+        <v>0</v>
+      </c>
+      <c r="H180" t="n">
+        <v>18</v>
+      </c>
+      <c r="I180" t="n">
+        <v>0</v>
+      </c>
+      <c r="J180" t="n">
+        <v>0</v>
+      </c>
+      <c r="K180" t="n">
+        <v>0</v>
+      </c>
+      <c r="L180" t="n">
+        <v>0</v>
+      </c>
+      <c r="M180" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F181" t="n">
+        <v>0</v>
+      </c>
+      <c r="G181" t="n">
+        <v>0</v>
+      </c>
+      <c r="H181" t="n">
+        <v>0</v>
+      </c>
+      <c r="I181" t="n">
+        <v>0</v>
+      </c>
+      <c r="J181" t="n">
+        <v>0</v>
+      </c>
+      <c r="K181" t="n">
+        <v>0</v>
+      </c>
+      <c r="L181" t="n">
+        <v>0</v>
+      </c>
+      <c r="M181" t="n">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M165"/>
+  <autoFilter ref="A1:M181"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8550,7 +9334,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G83"/>
+  <dimension ref="A1:G91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10916,12 +11700,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>PW</t>
+          <t>SMART BKK</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>LCHY5</t>
+          <t>BKK25</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -10930,13 +11714,13 @@
         </is>
       </c>
       <c r="E82" t="n">
-        <v>78</v>
+        <v>3</v>
       </c>
       <c r="F82" t="n">
-        <v>66</v>
+        <v>3</v>
       </c>
       <c r="G82" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="83">
@@ -10945,31 +11729,263 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
+          <t>SMART BKK</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>BKK25</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>13</v>
+      </c>
+      <c r="F83" t="n">
+        <v>13</v>
+      </c>
+      <c r="G83" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>BKK27</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>111</v>
+      </c>
+      <c r="F84" t="n">
+        <v>111</v>
+      </c>
+      <c r="G84" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>BKK27</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>46</v>
+      </c>
+      <c r="F85" t="n">
+        <v>46</v>
+      </c>
+      <c r="G85" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>HAST</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>LCH27</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>37</v>
+      </c>
+      <c r="F86" t="n">
+        <v>37</v>
+      </c>
+      <c r="G86" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>HAST</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>LCH27</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>30</v>
+      </c>
+      <c r="F87" t="n">
+        <v>30</v>
+      </c>
+      <c r="G87" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>LCH28</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>3</v>
+      </c>
+      <c r="F88" t="n">
+        <v>3</v>
+      </c>
+      <c r="G88" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>LCH28</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>2</v>
+      </c>
+      <c r="F89" t="n">
+        <v>2</v>
+      </c>
+      <c r="G89" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
           <t>PW</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr">
+      <c r="C90" t="inlineStr">
         <is>
           <t>LCHY5</t>
         </is>
       </c>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>GATE OUT</t>
-        </is>
-      </c>
-      <c r="E83" t="n">
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>78</v>
+      </c>
+      <c r="F90" t="n">
+        <v>78</v>
+      </c>
+      <c r="G90" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
         <v>44</v>
       </c>
-      <c r="F83" t="n">
-        <v>39</v>
-      </c>
-      <c r="G83" t="n">
-        <v>5</v>
+      <c r="F91" t="n">
+        <v>44</v>
+      </c>
+      <c r="G91" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G83"/>
+  <autoFilter ref="A1:G91"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
GATE IN: HAL#### / HAL##### and 15-char HASL? codes count as Agent; re-run all days
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gate-move-summary.xlsx
+++ b/docs/gate-move-summary.xlsx
@@ -4257,7 +4257,7 @@
         <v>0</v>
       </c>
       <c r="H78" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="I78" t="n">
         <v>0</v>
@@ -4272,7 +4272,7 @@
         <v>0</v>
       </c>
       <c r="M78" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="79">
@@ -4306,7 +4306,7 @@
         <v>0</v>
       </c>
       <c r="H79" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I79" t="n">
         <v>0</v>
@@ -4321,7 +4321,7 @@
         <v>0</v>
       </c>
       <c r="M79" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="80">
@@ -5231,7 +5231,7 @@
         </is>
       </c>
       <c r="F98" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="G98" t="n">
         <v>0</v>
@@ -5246,13 +5246,13 @@
         <v>0</v>
       </c>
       <c r="K98" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L98" t="n">
         <v>0</v>
       </c>
       <c r="M98" t="n">
-        <v>36</v>
+        <v>30</v>
       </c>
     </row>
     <row r="99">
@@ -5280,7 +5280,7 @@
         </is>
       </c>
       <c r="F99" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G99" t="n">
         <v>0</v>
@@ -5295,13 +5295,13 @@
         <v>0</v>
       </c>
       <c r="K99" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L99" t="n">
         <v>0</v>
       </c>
       <c r="M99" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="100">
@@ -6211,7 +6211,7 @@
         </is>
       </c>
       <c r="F118" t="n">
-        <v>51</v>
+        <v>3</v>
       </c>
       <c r="G118" t="n">
         <v>0</v>
@@ -6232,7 +6232,7 @@
         <v>0</v>
       </c>
       <c r="M118" t="n">
-        <v>60</v>
+        <v>12</v>
       </c>
     </row>
     <row r="119">
@@ -6260,7 +6260,7 @@
         </is>
       </c>
       <c r="F119" t="n">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="G119" t="n">
         <v>0</v>
@@ -6281,7 +6281,7 @@
         <v>0</v>
       </c>
       <c r="M119" t="n">
-        <v>1</v>
+        <v>49</v>
       </c>
     </row>
     <row r="120">
@@ -7191,7 +7191,7 @@
         </is>
       </c>
       <c r="F138" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="G138" t="n">
         <v>0</v>
@@ -7212,7 +7212,7 @@
         <v>0</v>
       </c>
       <c r="M138" t="n">
-        <v>37</v>
+        <v>29</v>
       </c>
     </row>
     <row r="139">
@@ -7240,7 +7240,7 @@
         </is>
       </c>
       <c r="F139" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G139" t="n">
         <v>0</v>
@@ -7261,7 +7261,7 @@
         <v>0</v>
       </c>
       <c r="M139" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="140">
@@ -9151,7 +9151,7 @@
         </is>
       </c>
       <c r="F178" t="n">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="G178" t="n">
         <v>0</v>
@@ -9172,7 +9172,7 @@
         <v>0</v>
       </c>
       <c r="M178" t="n">
-        <v>78</v>
+        <v>28</v>
       </c>
     </row>
     <row r="179">
@@ -9200,7 +9200,7 @@
         </is>
       </c>
       <c r="F179" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="G179" t="n">
         <v>0</v>
@@ -9221,7 +9221,7 @@
         <v>0</v>
       </c>
       <c r="M179" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="180">

</xml_diff>

<commit_message>
Add 22PC/42PC back (20'/40' FR); keep TPSZ column order in the database
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gate-move-summary.xlsx
+++ b/docs/gate-move-summary.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Compare" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daily Summary'!$A$1:$M$201</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daily Summary'!$A$1:$O$201</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'System Compare'!$A$1:$G$101</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M201"/>
+  <dimension ref="A1:O201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -498,6 +498,16 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>22PC</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>42PC</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>Total</t>
         </is>
       </c>
@@ -548,6 +558,12 @@
         <v>0</v>
       </c>
       <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
         <v>30</v>
       </c>
     </row>
@@ -599,6 +615,12 @@
       <c r="M3" t="n">
         <v>0</v>
       </c>
+      <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -646,6 +668,12 @@
         <v>0</v>
       </c>
       <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
         <v>7</v>
       </c>
     </row>
@@ -697,6 +725,12 @@
       <c r="M5" t="n">
         <v>0</v>
       </c>
+      <c r="N5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -744,6 +778,12 @@
         <v>0</v>
       </c>
       <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" t="n">
         <v>23</v>
       </c>
     </row>
@@ -795,6 +835,12 @@
       <c r="M7" t="n">
         <v>0</v>
       </c>
+      <c r="N7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -842,6 +888,12 @@
         <v>0</v>
       </c>
       <c r="M8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" t="n">
         <v>32</v>
       </c>
     </row>
@@ -891,6 +943,12 @@
         <v>0</v>
       </c>
       <c r="M9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" t="n">
         <v>18</v>
       </c>
     </row>
@@ -940,6 +998,12 @@
         <v>0</v>
       </c>
       <c r="M10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" t="n">
         <v>30</v>
       </c>
     </row>
@@ -989,6 +1053,12 @@
         <v>0</v>
       </c>
       <c r="M11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" t="n">
         <v>24</v>
       </c>
     </row>
@@ -1038,6 +1108,12 @@
         <v>0</v>
       </c>
       <c r="M12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" t="n">
         <v>22</v>
       </c>
     </row>
@@ -1089,6 +1165,12 @@
       <c r="M13" t="n">
         <v>0</v>
       </c>
+      <c r="N13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1138,6 +1220,12 @@
       <c r="M14" t="n">
         <v>0</v>
       </c>
+      <c r="N14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1187,6 +1275,12 @@
       <c r="M15" t="n">
         <v>0</v>
       </c>
+      <c r="N15" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1234,6 +1328,12 @@
         <v>0</v>
       </c>
       <c r="M16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" t="n">
         <v>9</v>
       </c>
     </row>
@@ -1285,6 +1385,12 @@
       <c r="M17" t="n">
         <v>0</v>
       </c>
+      <c r="N17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1332,6 +1438,12 @@
         <v>0</v>
       </c>
       <c r="M18" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" t="n">
         <v>42</v>
       </c>
     </row>
@@ -1381,6 +1493,12 @@
         <v>0</v>
       </c>
       <c r="M19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" t="n">
         <v>40</v>
       </c>
     </row>
@@ -1430,6 +1548,12 @@
         <v>0</v>
       </c>
       <c r="M20" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" t="n">
         <v>80</v>
       </c>
     </row>
@@ -1479,6 +1603,12 @@
         <v>0</v>
       </c>
       <c r="M21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1528,6 +1658,12 @@
         <v>0</v>
       </c>
       <c r="M22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" t="n">
         <v>38</v>
       </c>
     </row>
@@ -1579,6 +1715,12 @@
       <c r="M23" t="n">
         <v>0</v>
       </c>
+      <c r="N23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -1626,6 +1768,12 @@
         <v>0</v>
       </c>
       <c r="M24" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" t="n">
         <v>7</v>
       </c>
     </row>
@@ -1677,6 +1825,12 @@
       <c r="M25" t="n">
         <v>0</v>
       </c>
+      <c r="N25" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -1724,6 +1878,12 @@
         <v>0</v>
       </c>
       <c r="M26" t="n">
+        <v>0</v>
+      </c>
+      <c r="N26" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" t="n">
         <v>33</v>
       </c>
     </row>
@@ -1773,6 +1933,12 @@
         <v>0</v>
       </c>
       <c r="M27" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" t="n">
         <v>7</v>
       </c>
     </row>
@@ -1822,6 +1988,12 @@
         <v>0</v>
       </c>
       <c r="M28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" t="n">
         <v>74</v>
       </c>
     </row>
@@ -1873,6 +2045,12 @@
       <c r="M29" t="n">
         <v>0</v>
       </c>
+      <c r="N29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -1920,6 +2098,12 @@
         <v>0</v>
       </c>
       <c r="M30" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" t="n">
         <v>14</v>
       </c>
     </row>
@@ -1969,6 +2153,12 @@
         <v>0</v>
       </c>
       <c r="M31" t="n">
+        <v>0</v>
+      </c>
+      <c r="N31" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2018,6 +2208,12 @@
         <v>0</v>
       </c>
       <c r="M32" t="n">
+        <v>0</v>
+      </c>
+      <c r="N32" t="n">
+        <v>0</v>
+      </c>
+      <c r="O32" t="n">
         <v>5</v>
       </c>
     </row>
@@ -2067,6 +2263,12 @@
         <v>0</v>
       </c>
       <c r="M33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N33" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" t="n">
         <v>8</v>
       </c>
     </row>
@@ -2118,6 +2320,12 @@
       <c r="M34" t="n">
         <v>0</v>
       </c>
+      <c r="N34" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -2167,6 +2375,12 @@
       <c r="M35" t="n">
         <v>0</v>
       </c>
+      <c r="N35" t="n">
+        <v>0</v>
+      </c>
+      <c r="O35" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -2214,6 +2428,12 @@
         <v>0</v>
       </c>
       <c r="M36" t="n">
+        <v>0</v>
+      </c>
+      <c r="N36" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" t="n">
         <v>7</v>
       </c>
     </row>
@@ -2265,6 +2485,12 @@
       <c r="M37" t="n">
         <v>0</v>
       </c>
+      <c r="N37" t="n">
+        <v>0</v>
+      </c>
+      <c r="O37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -2312,6 +2538,12 @@
         <v>0</v>
       </c>
       <c r="M38" t="n">
+        <v>0</v>
+      </c>
+      <c r="N38" t="n">
+        <v>0</v>
+      </c>
+      <c r="O38" t="n">
         <v>41</v>
       </c>
     </row>
@@ -2361,6 +2593,12 @@
         <v>0</v>
       </c>
       <c r="M39" t="n">
+        <v>0</v>
+      </c>
+      <c r="N39" t="n">
+        <v>0</v>
+      </c>
+      <c r="O39" t="n">
         <v>23</v>
       </c>
     </row>
@@ -2410,6 +2648,12 @@
         <v>0</v>
       </c>
       <c r="M40" t="n">
+        <v>0</v>
+      </c>
+      <c r="N40" t="n">
+        <v>0</v>
+      </c>
+      <c r="O40" t="n">
         <v>33</v>
       </c>
     </row>
@@ -2461,6 +2705,12 @@
       <c r="M41" t="n">
         <v>0</v>
       </c>
+      <c r="N41" t="n">
+        <v>0</v>
+      </c>
+      <c r="O41" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -2508,6 +2758,12 @@
         <v>0</v>
       </c>
       <c r="M42" t="n">
+        <v>0</v>
+      </c>
+      <c r="N42" t="n">
+        <v>0</v>
+      </c>
+      <c r="O42" t="n">
         <v>18</v>
       </c>
     </row>
@@ -2559,6 +2815,12 @@
       <c r="M43" t="n">
         <v>0</v>
       </c>
+      <c r="N43" t="n">
+        <v>0</v>
+      </c>
+      <c r="O43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -2606,6 +2868,12 @@
         <v>0</v>
       </c>
       <c r="M44" t="n">
+        <v>0</v>
+      </c>
+      <c r="N44" t="n">
+        <v>0</v>
+      </c>
+      <c r="O44" t="n">
         <v>7</v>
       </c>
     </row>
@@ -2657,6 +2925,12 @@
       <c r="M45" t="n">
         <v>0</v>
       </c>
+      <c r="N45" t="n">
+        <v>0</v>
+      </c>
+      <c r="O45" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
@@ -2704,6 +2978,12 @@
         <v>0</v>
       </c>
       <c r="M46" t="n">
+        <v>0</v>
+      </c>
+      <c r="N46" t="n">
+        <v>0</v>
+      </c>
+      <c r="O46" t="n">
         <v>38</v>
       </c>
     </row>
@@ -2753,6 +3033,12 @@
         <v>0</v>
       </c>
       <c r="M47" t="n">
+        <v>0</v>
+      </c>
+      <c r="N47" t="n">
+        <v>0</v>
+      </c>
+      <c r="O47" t="n">
         <v>3</v>
       </c>
     </row>
@@ -2802,6 +3088,12 @@
         <v>0</v>
       </c>
       <c r="M48" t="n">
+        <v>0</v>
+      </c>
+      <c r="N48" t="n">
+        <v>0</v>
+      </c>
+      <c r="O48" t="n">
         <v>60</v>
       </c>
     </row>
@@ -2853,6 +3145,12 @@
       <c r="M49" t="n">
         <v>0</v>
       </c>
+      <c r="N49" t="n">
+        <v>0</v>
+      </c>
+      <c r="O49" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
@@ -2900,6 +3198,12 @@
         <v>0</v>
       </c>
       <c r="M50" t="n">
+        <v>0</v>
+      </c>
+      <c r="N50" t="n">
+        <v>0</v>
+      </c>
+      <c r="O50" t="n">
         <v>3</v>
       </c>
     </row>
@@ -2951,6 +3255,12 @@
       <c r="M51" t="n">
         <v>0</v>
       </c>
+      <c r="N51" t="n">
+        <v>0</v>
+      </c>
+      <c r="O51" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
@@ -2998,6 +3308,12 @@
         <v>0</v>
       </c>
       <c r="M52" t="n">
+        <v>0</v>
+      </c>
+      <c r="N52" t="n">
+        <v>0</v>
+      </c>
+      <c r="O52" t="n">
         <v>36</v>
       </c>
     </row>
@@ -3047,6 +3363,12 @@
         <v>0</v>
       </c>
       <c r="M53" t="n">
+        <v>0</v>
+      </c>
+      <c r="N53" t="n">
+        <v>0</v>
+      </c>
+      <c r="O53" t="n">
         <v>2</v>
       </c>
     </row>
@@ -3096,6 +3418,12 @@
         <v>0</v>
       </c>
       <c r="M54" t="n">
+        <v>0</v>
+      </c>
+      <c r="N54" t="n">
+        <v>0</v>
+      </c>
+      <c r="O54" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3147,6 +3475,12 @@
       <c r="M55" t="n">
         <v>0</v>
       </c>
+      <c r="N55" t="n">
+        <v>0</v>
+      </c>
+      <c r="O55" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
@@ -3194,6 +3528,12 @@
         <v>0</v>
       </c>
       <c r="M56" t="n">
+        <v>0</v>
+      </c>
+      <c r="N56" t="n">
+        <v>0</v>
+      </c>
+      <c r="O56" t="n">
         <v>4</v>
       </c>
     </row>
@@ -3245,6 +3585,12 @@
       <c r="M57" t="n">
         <v>0</v>
       </c>
+      <c r="N57" t="n">
+        <v>0</v>
+      </c>
+      <c r="O57" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
@@ -3292,6 +3638,12 @@
         <v>0</v>
       </c>
       <c r="M58" t="n">
+        <v>0</v>
+      </c>
+      <c r="N58" t="n">
+        <v>0</v>
+      </c>
+      <c r="O58" t="n">
         <v>49</v>
       </c>
     </row>
@@ -3341,6 +3693,12 @@
         <v>0</v>
       </c>
       <c r="M59" t="n">
+        <v>0</v>
+      </c>
+      <c r="N59" t="n">
+        <v>0</v>
+      </c>
+      <c r="O59" t="n">
         <v>16</v>
       </c>
     </row>
@@ -3390,6 +3748,12 @@
         <v>0</v>
       </c>
       <c r="M60" t="n">
+        <v>0</v>
+      </c>
+      <c r="N60" t="n">
+        <v>0</v>
+      </c>
+      <c r="O60" t="n">
         <v>36</v>
       </c>
     </row>
@@ -3439,6 +3803,12 @@
         <v>0</v>
       </c>
       <c r="M61" t="n">
+        <v>0</v>
+      </c>
+      <c r="N61" t="n">
+        <v>0</v>
+      </c>
+      <c r="O61" t="n">
         <v>2</v>
       </c>
     </row>
@@ -3488,6 +3858,12 @@
         <v>0</v>
       </c>
       <c r="M62" t="n">
+        <v>0</v>
+      </c>
+      <c r="N62" t="n">
+        <v>0</v>
+      </c>
+      <c r="O62" t="n">
         <v>23</v>
       </c>
     </row>
@@ -3539,6 +3915,12 @@
       <c r="M63" t="n">
         <v>0</v>
       </c>
+      <c r="N63" t="n">
+        <v>0</v>
+      </c>
+      <c r="O63" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
@@ -3586,6 +3968,12 @@
         <v>0</v>
       </c>
       <c r="M64" t="n">
+        <v>0</v>
+      </c>
+      <c r="N64" t="n">
+        <v>0</v>
+      </c>
+      <c r="O64" t="n">
         <v>6</v>
       </c>
     </row>
@@ -3637,6 +4025,12 @@
       <c r="M65" t="n">
         <v>0</v>
       </c>
+      <c r="N65" t="n">
+        <v>0</v>
+      </c>
+      <c r="O65" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
@@ -3684,6 +4078,12 @@
         <v>0</v>
       </c>
       <c r="M66" t="n">
+        <v>0</v>
+      </c>
+      <c r="N66" t="n">
+        <v>0</v>
+      </c>
+      <c r="O66" t="n">
         <v>18</v>
       </c>
     </row>
@@ -3735,6 +4135,12 @@
       <c r="M67" t="n">
         <v>0</v>
       </c>
+      <c r="N67" t="n">
+        <v>0</v>
+      </c>
+      <c r="O67" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
@@ -3782,6 +4188,12 @@
         <v>0</v>
       </c>
       <c r="M68" t="n">
+        <v>0</v>
+      </c>
+      <c r="N68" t="n">
+        <v>0</v>
+      </c>
+      <c r="O68" t="n">
         <v>57</v>
       </c>
     </row>
@@ -3831,6 +4243,12 @@
         <v>0</v>
       </c>
       <c r="M69" t="n">
+        <v>0</v>
+      </c>
+      <c r="N69" t="n">
+        <v>0</v>
+      </c>
+      <c r="O69" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3880,6 +4298,12 @@
         <v>0</v>
       </c>
       <c r="M70" t="n">
+        <v>0</v>
+      </c>
+      <c r="N70" t="n">
+        <v>0</v>
+      </c>
+      <c r="O70" t="n">
         <v>31</v>
       </c>
     </row>
@@ -3929,6 +4353,12 @@
         <v>0</v>
       </c>
       <c r="M71" t="n">
+        <v>0</v>
+      </c>
+      <c r="N71" t="n">
+        <v>0</v>
+      </c>
+      <c r="O71" t="n">
         <v>2</v>
       </c>
     </row>
@@ -3978,6 +4408,12 @@
         <v>0</v>
       </c>
       <c r="M72" t="n">
+        <v>0</v>
+      </c>
+      <c r="N72" t="n">
+        <v>0</v>
+      </c>
+      <c r="O72" t="n">
         <v>19</v>
       </c>
     </row>
@@ -4029,6 +4465,12 @@
       <c r="M73" t="n">
         <v>0</v>
       </c>
+      <c r="N73" t="n">
+        <v>0</v>
+      </c>
+      <c r="O73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
@@ -4078,6 +4520,12 @@
       <c r="M74" t="n">
         <v>0</v>
       </c>
+      <c r="N74" t="n">
+        <v>0</v>
+      </c>
+      <c r="O74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
@@ -4127,6 +4575,12 @@
       <c r="M75" t="n">
         <v>0</v>
       </c>
+      <c r="N75" t="n">
+        <v>0</v>
+      </c>
+      <c r="O75" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
@@ -4174,6 +4628,12 @@
         <v>0</v>
       </c>
       <c r="M76" t="n">
+        <v>0</v>
+      </c>
+      <c r="N76" t="n">
+        <v>0</v>
+      </c>
+      <c r="O76" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4225,6 +4685,12 @@
       <c r="M77" t="n">
         <v>0</v>
       </c>
+      <c r="N77" t="n">
+        <v>0</v>
+      </c>
+      <c r="O77" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
@@ -4272,6 +4738,12 @@
         <v>0</v>
       </c>
       <c r="M78" t="n">
+        <v>0</v>
+      </c>
+      <c r="N78" t="n">
+        <v>0</v>
+      </c>
+      <c r="O78" t="n">
         <v>42</v>
       </c>
     </row>
@@ -4321,6 +4793,12 @@
         <v>0</v>
       </c>
       <c r="M79" t="n">
+        <v>0</v>
+      </c>
+      <c r="N79" t="n">
+        <v>0</v>
+      </c>
+      <c r="O79" t="n">
         <v>14</v>
       </c>
     </row>
@@ -4370,6 +4848,12 @@
         <v>0</v>
       </c>
       <c r="M80" t="n">
+        <v>0</v>
+      </c>
+      <c r="N80" t="n">
+        <v>0</v>
+      </c>
+      <c r="O80" t="n">
         <v>64</v>
       </c>
     </row>
@@ -4419,6 +4903,12 @@
         <v>0</v>
       </c>
       <c r="M81" t="n">
+        <v>0</v>
+      </c>
+      <c r="N81" t="n">
+        <v>0</v>
+      </c>
+      <c r="O81" t="n">
         <v>4</v>
       </c>
     </row>
@@ -4468,6 +4958,12 @@
         <v>0</v>
       </c>
       <c r="M82" t="n">
+        <v>0</v>
+      </c>
+      <c r="N82" t="n">
+        <v>0</v>
+      </c>
+      <c r="O82" t="n">
         <v>19</v>
       </c>
     </row>
@@ -4519,6 +5015,12 @@
       <c r="M83" t="n">
         <v>0</v>
       </c>
+      <c r="N83" t="n">
+        <v>0</v>
+      </c>
+      <c r="O83" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
@@ -4566,6 +5068,12 @@
         <v>0</v>
       </c>
       <c r="M84" t="n">
+        <v>0</v>
+      </c>
+      <c r="N84" t="n">
+        <v>0</v>
+      </c>
+      <c r="O84" t="n">
         <v>3</v>
       </c>
     </row>
@@ -4617,6 +5125,12 @@
       <c r="M85" t="n">
         <v>0</v>
       </c>
+      <c r="N85" t="n">
+        <v>0</v>
+      </c>
+      <c r="O85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
@@ -4664,6 +5178,12 @@
         <v>0</v>
       </c>
       <c r="M86" t="n">
+        <v>0</v>
+      </c>
+      <c r="N86" t="n">
+        <v>0</v>
+      </c>
+      <c r="O86" t="n">
         <v>22</v>
       </c>
     </row>
@@ -4715,6 +5235,12 @@
       <c r="M87" t="n">
         <v>0</v>
       </c>
+      <c r="N87" t="n">
+        <v>0</v>
+      </c>
+      <c r="O87" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
@@ -4762,6 +5288,12 @@
         <v>0</v>
       </c>
       <c r="M88" t="n">
+        <v>0</v>
+      </c>
+      <c r="N88" t="n">
+        <v>0</v>
+      </c>
+      <c r="O88" t="n">
         <v>23</v>
       </c>
     </row>
@@ -4811,6 +5343,12 @@
         <v>0</v>
       </c>
       <c r="M89" t="n">
+        <v>0</v>
+      </c>
+      <c r="N89" t="n">
+        <v>0</v>
+      </c>
+      <c r="O89" t="n">
         <v>8</v>
       </c>
     </row>
@@ -4860,6 +5398,12 @@
         <v>0</v>
       </c>
       <c r="M90" t="n">
+        <v>0</v>
+      </c>
+      <c r="N90" t="n">
+        <v>0</v>
+      </c>
+      <c r="O90" t="n">
         <v>18</v>
       </c>
     </row>
@@ -4909,6 +5453,12 @@
         <v>0</v>
       </c>
       <c r="M91" t="n">
+        <v>0</v>
+      </c>
+      <c r="N91" t="n">
+        <v>0</v>
+      </c>
+      <c r="O91" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4958,6 +5508,12 @@
         <v>0</v>
       </c>
       <c r="M92" t="n">
+        <v>0</v>
+      </c>
+      <c r="N92" t="n">
+        <v>0</v>
+      </c>
+      <c r="O92" t="n">
         <v>17</v>
       </c>
     </row>
@@ -5009,6 +5565,12 @@
       <c r="M93" t="n">
         <v>0</v>
       </c>
+      <c r="N93" t="n">
+        <v>0</v>
+      </c>
+      <c r="O93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
@@ -5056,6 +5618,12 @@
         <v>0</v>
       </c>
       <c r="M94" t="n">
+        <v>0</v>
+      </c>
+      <c r="N94" t="n">
+        <v>0</v>
+      </c>
+      <c r="O94" t="n">
         <v>2</v>
       </c>
     </row>
@@ -5107,6 +5675,12 @@
       <c r="M95" t="n">
         <v>0</v>
       </c>
+      <c r="N95" t="n">
+        <v>0</v>
+      </c>
+      <c r="O95" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
@@ -5154,6 +5728,12 @@
         <v>0</v>
       </c>
       <c r="M96" t="n">
+        <v>0</v>
+      </c>
+      <c r="N96" t="n">
+        <v>0</v>
+      </c>
+      <c r="O96" t="n">
         <v>3</v>
       </c>
     </row>
@@ -5205,6 +5785,12 @@
       <c r="M97" t="n">
         <v>0</v>
       </c>
+      <c r="N97" t="n">
+        <v>0</v>
+      </c>
+      <c r="O97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
@@ -5252,6 +5838,12 @@
         <v>0</v>
       </c>
       <c r="M98" t="n">
+        <v>0</v>
+      </c>
+      <c r="N98" t="n">
+        <v>0</v>
+      </c>
+      <c r="O98" t="n">
         <v>30</v>
       </c>
     </row>
@@ -5301,6 +5893,12 @@
         <v>0</v>
       </c>
       <c r="M99" t="n">
+        <v>0</v>
+      </c>
+      <c r="N99" t="n">
+        <v>0</v>
+      </c>
+      <c r="O99" t="n">
         <v>7</v>
       </c>
     </row>
@@ -5350,6 +5948,12 @@
         <v>0</v>
       </c>
       <c r="M100" t="n">
+        <v>0</v>
+      </c>
+      <c r="N100" t="n">
+        <v>0</v>
+      </c>
+      <c r="O100" t="n">
         <v>25</v>
       </c>
     </row>
@@ -5401,6 +6005,12 @@
       <c r="M101" t="n">
         <v>0</v>
       </c>
+      <c r="N101" t="n">
+        <v>0</v>
+      </c>
+      <c r="O101" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
@@ -5448,6 +6058,12 @@
         <v>0</v>
       </c>
       <c r="M102" t="n">
+        <v>0</v>
+      </c>
+      <c r="N102" t="n">
+        <v>0</v>
+      </c>
+      <c r="O102" t="n">
         <v>7</v>
       </c>
     </row>
@@ -5499,6 +6115,12 @@
       <c r="M103" t="n">
         <v>0</v>
       </c>
+      <c r="N103" t="n">
+        <v>0</v>
+      </c>
+      <c r="O103" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
@@ -5546,6 +6168,12 @@
         <v>0</v>
       </c>
       <c r="M104" t="n">
+        <v>0</v>
+      </c>
+      <c r="N104" t="n">
+        <v>0</v>
+      </c>
+      <c r="O104" t="n">
         <v>16</v>
       </c>
     </row>
@@ -5597,6 +6225,12 @@
       <c r="M105" t="n">
         <v>0</v>
       </c>
+      <c r="N105" t="n">
+        <v>0</v>
+      </c>
+      <c r="O105" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
@@ -5644,6 +6278,12 @@
         <v>0</v>
       </c>
       <c r="M106" t="n">
+        <v>0</v>
+      </c>
+      <c r="N106" t="n">
+        <v>0</v>
+      </c>
+      <c r="O106" t="n">
         <v>44</v>
       </c>
     </row>
@@ -5695,6 +6335,12 @@
       <c r="M107" t="n">
         <v>0</v>
       </c>
+      <c r="N107" t="n">
+        <v>0</v>
+      </c>
+      <c r="O107" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
@@ -5742,6 +6388,12 @@
         <v>0</v>
       </c>
       <c r="M108" t="n">
+        <v>0</v>
+      </c>
+      <c r="N108" t="n">
+        <v>0</v>
+      </c>
+      <c r="O108" t="n">
         <v>22</v>
       </c>
     </row>
@@ -5793,6 +6445,12 @@
       <c r="M109" t="n">
         <v>0</v>
       </c>
+      <c r="N109" t="n">
+        <v>0</v>
+      </c>
+      <c r="O109" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
@@ -5840,6 +6498,12 @@
         <v>0</v>
       </c>
       <c r="M110" t="n">
+        <v>0</v>
+      </c>
+      <c r="N110" t="n">
+        <v>0</v>
+      </c>
+      <c r="O110" t="n">
         <v>22</v>
       </c>
     </row>
@@ -5889,6 +6553,12 @@
         <v>0</v>
       </c>
       <c r="M111" t="n">
+        <v>0</v>
+      </c>
+      <c r="N111" t="n">
+        <v>0</v>
+      </c>
+      <c r="O111" t="n">
         <v>6</v>
       </c>
     </row>
@@ -5938,6 +6608,12 @@
         <v>0</v>
       </c>
       <c r="M112" t="n">
+        <v>0</v>
+      </c>
+      <c r="N112" t="n">
+        <v>0</v>
+      </c>
+      <c r="O112" t="n">
         <v>15</v>
       </c>
     </row>
@@ -5987,6 +6663,12 @@
         <v>0</v>
       </c>
       <c r="M113" t="n">
+        <v>0</v>
+      </c>
+      <c r="N113" t="n">
+        <v>0</v>
+      </c>
+      <c r="O113" t="n">
         <v>4</v>
       </c>
     </row>
@@ -6036,6 +6718,12 @@
         <v>0</v>
       </c>
       <c r="M114" t="n">
+        <v>0</v>
+      </c>
+      <c r="N114" t="n">
+        <v>0</v>
+      </c>
+      <c r="O114" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6087,6 +6775,12 @@
       <c r="M115" t="n">
         <v>0</v>
       </c>
+      <c r="N115" t="n">
+        <v>0</v>
+      </c>
+      <c r="O115" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
@@ -6136,6 +6830,12 @@
       <c r="M116" t="n">
         <v>0</v>
       </c>
+      <c r="N116" t="n">
+        <v>0</v>
+      </c>
+      <c r="O116" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
@@ -6185,6 +6885,12 @@
       <c r="M117" t="n">
         <v>0</v>
       </c>
+      <c r="N117" t="n">
+        <v>0</v>
+      </c>
+      <c r="O117" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
@@ -6232,6 +6938,12 @@
         <v>0</v>
       </c>
       <c r="M118" t="n">
+        <v>0</v>
+      </c>
+      <c r="N118" t="n">
+        <v>0</v>
+      </c>
+      <c r="O118" t="n">
         <v>12</v>
       </c>
     </row>
@@ -6281,6 +6993,12 @@
         <v>0</v>
       </c>
       <c r="M119" t="n">
+        <v>0</v>
+      </c>
+      <c r="N119" t="n">
+        <v>0</v>
+      </c>
+      <c r="O119" t="n">
         <v>49</v>
       </c>
     </row>
@@ -6330,6 +7048,12 @@
         <v>0</v>
       </c>
       <c r="M120" t="n">
+        <v>0</v>
+      </c>
+      <c r="N120" t="n">
+        <v>0</v>
+      </c>
+      <c r="O120" t="n">
         <v>36</v>
       </c>
     </row>
@@ -6381,6 +7105,12 @@
       <c r="M121" t="n">
         <v>0</v>
       </c>
+      <c r="N121" t="n">
+        <v>0</v>
+      </c>
+      <c r="O121" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="n">
@@ -6428,6 +7158,12 @@
         <v>0</v>
       </c>
       <c r="M122" t="n">
+        <v>0</v>
+      </c>
+      <c r="N122" t="n">
+        <v>0</v>
+      </c>
+      <c r="O122" t="n">
         <v>10</v>
       </c>
     </row>
@@ -6479,6 +7215,12 @@
       <c r="M123" t="n">
         <v>0</v>
       </c>
+      <c r="N123" t="n">
+        <v>0</v>
+      </c>
+      <c r="O123" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="n">
@@ -6526,6 +7268,12 @@
         <v>0</v>
       </c>
       <c r="M124" t="n">
+        <v>0</v>
+      </c>
+      <c r="N124" t="n">
+        <v>0</v>
+      </c>
+      <c r="O124" t="n">
         <v>3</v>
       </c>
     </row>
@@ -6577,6 +7325,12 @@
       <c r="M125" t="n">
         <v>0</v>
       </c>
+      <c r="N125" t="n">
+        <v>0</v>
+      </c>
+      <c r="O125" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="n">
@@ -6624,6 +7378,12 @@
         <v>0</v>
       </c>
       <c r="M126" t="n">
+        <v>0</v>
+      </c>
+      <c r="N126" t="n">
+        <v>0</v>
+      </c>
+      <c r="O126" t="n">
         <v>65</v>
       </c>
     </row>
@@ -6675,6 +7435,12 @@
       <c r="M127" t="n">
         <v>0</v>
       </c>
+      <c r="N127" t="n">
+        <v>0</v>
+      </c>
+      <c r="O127" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="n">
@@ -6722,6 +7488,12 @@
         <v>0</v>
       </c>
       <c r="M128" t="n">
+        <v>0</v>
+      </c>
+      <c r="N128" t="n">
+        <v>0</v>
+      </c>
+      <c r="O128" t="n">
         <v>35</v>
       </c>
     </row>
@@ -6771,6 +7543,12 @@
         <v>0</v>
       </c>
       <c r="M129" t="n">
+        <v>0</v>
+      </c>
+      <c r="N129" t="n">
+        <v>0</v>
+      </c>
+      <c r="O129" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6820,6 +7598,12 @@
         <v>0</v>
       </c>
       <c r="M130" t="n">
+        <v>0</v>
+      </c>
+      <c r="N130" t="n">
+        <v>0</v>
+      </c>
+      <c r="O130" t="n">
         <v>23</v>
       </c>
     </row>
@@ -6869,6 +7653,12 @@
         <v>0</v>
       </c>
       <c r="M131" t="n">
+        <v>0</v>
+      </c>
+      <c r="N131" t="n">
+        <v>0</v>
+      </c>
+      <c r="O131" t="n">
         <v>16</v>
       </c>
     </row>
@@ -6918,6 +7708,12 @@
         <v>0</v>
       </c>
       <c r="M132" t="n">
+        <v>0</v>
+      </c>
+      <c r="N132" t="n">
+        <v>0</v>
+      </c>
+      <c r="O132" t="n">
         <v>7</v>
       </c>
     </row>
@@ -6967,6 +7763,12 @@
         <v>0</v>
       </c>
       <c r="M133" t="n">
+        <v>0</v>
+      </c>
+      <c r="N133" t="n">
+        <v>0</v>
+      </c>
+      <c r="O133" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7016,6 +7818,12 @@
         <v>0</v>
       </c>
       <c r="M134" t="n">
+        <v>0</v>
+      </c>
+      <c r="N134" t="n">
+        <v>0</v>
+      </c>
+      <c r="O134" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7067,6 +7875,12 @@
       <c r="M135" t="n">
         <v>0</v>
       </c>
+      <c r="N135" t="n">
+        <v>0</v>
+      </c>
+      <c r="O135" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="n">
@@ -7114,6 +7928,12 @@
         <v>0</v>
       </c>
       <c r="M136" t="n">
+        <v>0</v>
+      </c>
+      <c r="N136" t="n">
+        <v>0</v>
+      </c>
+      <c r="O136" t="n">
         <v>3</v>
       </c>
     </row>
@@ -7165,6 +7985,12 @@
       <c r="M137" t="n">
         <v>0</v>
       </c>
+      <c r="N137" t="n">
+        <v>0</v>
+      </c>
+      <c r="O137" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="n">
@@ -7212,6 +8038,12 @@
         <v>0</v>
       </c>
       <c r="M138" t="n">
+        <v>0</v>
+      </c>
+      <c r="N138" t="n">
+        <v>0</v>
+      </c>
+      <c r="O138" t="n">
         <v>29</v>
       </c>
     </row>
@@ -7261,6 +8093,12 @@
         <v>0</v>
       </c>
       <c r="M139" t="n">
+        <v>0</v>
+      </c>
+      <c r="N139" t="n">
+        <v>0</v>
+      </c>
+      <c r="O139" t="n">
         <v>8</v>
       </c>
     </row>
@@ -7310,6 +8148,12 @@
         <v>0</v>
       </c>
       <c r="M140" t="n">
+        <v>0</v>
+      </c>
+      <c r="N140" t="n">
+        <v>0</v>
+      </c>
+      <c r="O140" t="n">
         <v>34</v>
       </c>
     </row>
@@ -7361,6 +8205,12 @@
       <c r="M141" t="n">
         <v>0</v>
       </c>
+      <c r="N141" t="n">
+        <v>0</v>
+      </c>
+      <c r="O141" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="n">
@@ -7408,6 +8258,12 @@
         <v>0</v>
       </c>
       <c r="M142" t="n">
+        <v>0</v>
+      </c>
+      <c r="N142" t="n">
+        <v>0</v>
+      </c>
+      <c r="O142" t="n">
         <v>5</v>
       </c>
     </row>
@@ -7459,6 +8315,12 @@
       <c r="M143" t="n">
         <v>0</v>
       </c>
+      <c r="N143" t="n">
+        <v>0</v>
+      </c>
+      <c r="O143" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="n">
@@ -7506,6 +8368,12 @@
         <v>0</v>
       </c>
       <c r="M144" t="n">
+        <v>0</v>
+      </c>
+      <c r="N144" t="n">
+        <v>0</v>
+      </c>
+      <c r="O144" t="n">
         <v>11</v>
       </c>
     </row>
@@ -7557,6 +8425,12 @@
       <c r="M145" t="n">
         <v>0</v>
       </c>
+      <c r="N145" t="n">
+        <v>0</v>
+      </c>
+      <c r="O145" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="n">
@@ -7604,6 +8478,12 @@
         <v>0</v>
       </c>
       <c r="M146" t="n">
+        <v>0</v>
+      </c>
+      <c r="N146" t="n">
+        <v>0</v>
+      </c>
+      <c r="O146" t="n">
         <v>105</v>
       </c>
     </row>
@@ -7655,6 +8535,12 @@
       <c r="M147" t="n">
         <v>0</v>
       </c>
+      <c r="N147" t="n">
+        <v>0</v>
+      </c>
+      <c r="O147" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="n">
@@ -7702,6 +8588,12 @@
         <v>0</v>
       </c>
       <c r="M148" t="n">
+        <v>0</v>
+      </c>
+      <c r="N148" t="n">
+        <v>0</v>
+      </c>
+      <c r="O148" t="n">
         <v>76</v>
       </c>
     </row>
@@ -7753,6 +8645,12 @@
       <c r="M149" t="n">
         <v>0</v>
       </c>
+      <c r="N149" t="n">
+        <v>0</v>
+      </c>
+      <c r="O149" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="n">
@@ -7800,6 +8698,12 @@
         <v>0</v>
       </c>
       <c r="M150" t="n">
+        <v>0</v>
+      </c>
+      <c r="N150" t="n">
+        <v>0</v>
+      </c>
+      <c r="O150" t="n">
         <v>23</v>
       </c>
     </row>
@@ -7849,6 +8753,12 @@
         <v>0</v>
       </c>
       <c r="M151" t="n">
+        <v>0</v>
+      </c>
+      <c r="N151" t="n">
+        <v>0</v>
+      </c>
+      <c r="O151" t="n">
         <v>5</v>
       </c>
     </row>
@@ -7898,6 +8808,12 @@
         <v>0</v>
       </c>
       <c r="M152" t="n">
+        <v>0</v>
+      </c>
+      <c r="N152" t="n">
+        <v>0</v>
+      </c>
+      <c r="O152" t="n">
         <v>16</v>
       </c>
     </row>
@@ -7949,6 +8865,12 @@
       <c r="M153" t="n">
         <v>0</v>
       </c>
+      <c r="N153" t="n">
+        <v>0</v>
+      </c>
+      <c r="O153" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="n">
@@ -7996,6 +8918,12 @@
         <v>0</v>
       </c>
       <c r="M154" t="n">
+        <v>0</v>
+      </c>
+      <c r="N154" t="n">
+        <v>0</v>
+      </c>
+      <c r="O154" t="n">
         <v>1</v>
       </c>
     </row>
@@ -8047,6 +8975,12 @@
       <c r="M155" t="n">
         <v>0</v>
       </c>
+      <c r="N155" t="n">
+        <v>0</v>
+      </c>
+      <c r="O155" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="n">
@@ -8096,6 +9030,12 @@
       <c r="M156" t="n">
         <v>0</v>
       </c>
+      <c r="N156" t="n">
+        <v>0</v>
+      </c>
+      <c r="O156" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="n">
@@ -8145,6 +9085,12 @@
       <c r="M157" t="n">
         <v>0</v>
       </c>
+      <c r="N157" t="n">
+        <v>0</v>
+      </c>
+      <c r="O157" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="n">
@@ -8192,6 +9138,12 @@
         <v>0</v>
       </c>
       <c r="M158" t="n">
+        <v>0</v>
+      </c>
+      <c r="N158" t="n">
+        <v>0</v>
+      </c>
+      <c r="O158" t="n">
         <v>36</v>
       </c>
     </row>
@@ -8243,6 +9195,12 @@
       <c r="M159" t="n">
         <v>0</v>
       </c>
+      <c r="N159" t="n">
+        <v>0</v>
+      </c>
+      <c r="O159" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="n">
@@ -8290,6 +9248,12 @@
         <v>0</v>
       </c>
       <c r="M160" t="n">
+        <v>0</v>
+      </c>
+      <c r="N160" t="n">
+        <v>0</v>
+      </c>
+      <c r="O160" t="n">
         <v>36</v>
       </c>
     </row>
@@ -8339,6 +9303,12 @@
         <v>0</v>
       </c>
       <c r="M161" t="n">
+        <v>0</v>
+      </c>
+      <c r="N161" t="n">
+        <v>0</v>
+      </c>
+      <c r="O161" t="n">
         <v>1</v>
       </c>
     </row>
@@ -8388,6 +9358,12 @@
         <v>0</v>
       </c>
       <c r="M162" t="n">
+        <v>0</v>
+      </c>
+      <c r="N162" t="n">
+        <v>0</v>
+      </c>
+      <c r="O162" t="n">
         <v>3</v>
       </c>
     </row>
@@ -8439,6 +9415,12 @@
       <c r="M163" t="n">
         <v>0</v>
       </c>
+      <c r="N163" t="n">
+        <v>0</v>
+      </c>
+      <c r="O163" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="n">
@@ -8486,6 +9468,12 @@
         <v>0</v>
       </c>
       <c r="M164" t="n">
+        <v>0</v>
+      </c>
+      <c r="N164" t="n">
+        <v>0</v>
+      </c>
+      <c r="O164" t="n">
         <v>13</v>
       </c>
     </row>
@@ -8537,6 +9525,12 @@
       <c r="M165" t="n">
         <v>0</v>
       </c>
+      <c r="N165" t="n">
+        <v>0</v>
+      </c>
+      <c r="O165" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="n">
@@ -8584,6 +9578,12 @@
         <v>0</v>
       </c>
       <c r="M166" t="n">
+        <v>0</v>
+      </c>
+      <c r="N166" t="n">
+        <v>0</v>
+      </c>
+      <c r="O166" t="n">
         <v>103</v>
       </c>
     </row>
@@ -8633,6 +9633,12 @@
         <v>0</v>
       </c>
       <c r="M167" t="n">
+        <v>0</v>
+      </c>
+      <c r="N167" t="n">
+        <v>0</v>
+      </c>
+      <c r="O167" t="n">
         <v>8</v>
       </c>
     </row>
@@ -8682,6 +9688,12 @@
         <v>0</v>
       </c>
       <c r="M168" t="n">
+        <v>0</v>
+      </c>
+      <c r="N168" t="n">
+        <v>0</v>
+      </c>
+      <c r="O168" t="n">
         <v>45</v>
       </c>
     </row>
@@ -8731,6 +9743,12 @@
         <v>0</v>
       </c>
       <c r="M169" t="n">
+        <v>0</v>
+      </c>
+      <c r="N169" t="n">
+        <v>0</v>
+      </c>
+      <c r="O169" t="n">
         <v>1</v>
       </c>
     </row>
@@ -8780,6 +9798,12 @@
         <v>0</v>
       </c>
       <c r="M170" t="n">
+        <v>0</v>
+      </c>
+      <c r="N170" t="n">
+        <v>0</v>
+      </c>
+      <c r="O170" t="n">
         <v>29</v>
       </c>
     </row>
@@ -8829,6 +9853,12 @@
         <v>0</v>
       </c>
       <c r="M171" t="n">
+        <v>0</v>
+      </c>
+      <c r="N171" t="n">
+        <v>0</v>
+      </c>
+      <c r="O171" t="n">
         <v>8</v>
       </c>
     </row>
@@ -8878,6 +9908,12 @@
         <v>0</v>
       </c>
       <c r="M172" t="n">
+        <v>0</v>
+      </c>
+      <c r="N172" t="n">
+        <v>0</v>
+      </c>
+      <c r="O172" t="n">
         <v>26</v>
       </c>
     </row>
@@ -8927,6 +9963,12 @@
         <v>0</v>
       </c>
       <c r="M173" t="n">
+        <v>0</v>
+      </c>
+      <c r="N173" t="n">
+        <v>0</v>
+      </c>
+      <c r="O173" t="n">
         <v>4</v>
       </c>
     </row>
@@ -8976,6 +10018,12 @@
         <v>0</v>
       </c>
       <c r="M174" t="n">
+        <v>0</v>
+      </c>
+      <c r="N174" t="n">
+        <v>0</v>
+      </c>
+      <c r="O174" t="n">
         <v>3</v>
       </c>
     </row>
@@ -9027,6 +10075,12 @@
       <c r="M175" t="n">
         <v>0</v>
       </c>
+      <c r="N175" t="n">
+        <v>0</v>
+      </c>
+      <c r="O175" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="n">
@@ -9074,6 +10128,12 @@
         <v>0</v>
       </c>
       <c r="M176" t="n">
+        <v>0</v>
+      </c>
+      <c r="N176" t="n">
+        <v>0</v>
+      </c>
+      <c r="O176" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9123,6 +10183,12 @@
         <v>0</v>
       </c>
       <c r="M177" t="n">
+        <v>0</v>
+      </c>
+      <c r="N177" t="n">
+        <v>0</v>
+      </c>
+      <c r="O177" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9172,6 +10238,12 @@
         <v>0</v>
       </c>
       <c r="M178" t="n">
+        <v>0</v>
+      </c>
+      <c r="N178" t="n">
+        <v>0</v>
+      </c>
+      <c r="O178" t="n">
         <v>28</v>
       </c>
     </row>
@@ -9221,6 +10293,12 @@
         <v>0</v>
       </c>
       <c r="M179" t="n">
+        <v>0</v>
+      </c>
+      <c r="N179" t="n">
+        <v>0</v>
+      </c>
+      <c r="O179" t="n">
         <v>50</v>
       </c>
     </row>
@@ -9270,6 +10348,12 @@
         <v>0</v>
       </c>
       <c r="M180" t="n">
+        <v>0</v>
+      </c>
+      <c r="N180" t="n">
+        <v>0</v>
+      </c>
+      <c r="O180" t="n">
         <v>44</v>
       </c>
     </row>
@@ -9321,6 +10405,12 @@
       <c r="M181" t="n">
         <v>0</v>
       </c>
+      <c r="N181" t="n">
+        <v>0</v>
+      </c>
+      <c r="O181" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="n">
@@ -9368,6 +10458,12 @@
         <v>0</v>
       </c>
       <c r="M182" t="n">
+        <v>0</v>
+      </c>
+      <c r="N182" t="n">
+        <v>0</v>
+      </c>
+      <c r="O182" t="n">
         <v>7</v>
       </c>
     </row>
@@ -9419,6 +10515,12 @@
       <c r="M183" t="n">
         <v>0</v>
       </c>
+      <c r="N183" t="n">
+        <v>0</v>
+      </c>
+      <c r="O183" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="n">
@@ -9466,6 +10568,12 @@
         <v>0</v>
       </c>
       <c r="M184" t="n">
+        <v>0</v>
+      </c>
+      <c r="N184" t="n">
+        <v>0</v>
+      </c>
+      <c r="O184" t="n">
         <v>29</v>
       </c>
     </row>
@@ -9517,6 +10625,12 @@
       <c r="M185" t="n">
         <v>0</v>
       </c>
+      <c r="N185" t="n">
+        <v>0</v>
+      </c>
+      <c r="O185" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="n">
@@ -9564,6 +10678,12 @@
         <v>0</v>
       </c>
       <c r="M186" t="n">
+        <v>0</v>
+      </c>
+      <c r="N186" t="n">
+        <v>0</v>
+      </c>
+      <c r="O186" t="n">
         <v>69</v>
       </c>
     </row>
@@ -9613,6 +10733,12 @@
         <v>0</v>
       </c>
       <c r="M187" t="n">
+        <v>0</v>
+      </c>
+      <c r="N187" t="n">
+        <v>0</v>
+      </c>
+      <c r="O187" t="n">
         <v>31</v>
       </c>
     </row>
@@ -9662,6 +10788,12 @@
         <v>0</v>
       </c>
       <c r="M188" t="n">
+        <v>0</v>
+      </c>
+      <c r="N188" t="n">
+        <v>0</v>
+      </c>
+      <c r="O188" t="n">
         <v>104</v>
       </c>
     </row>
@@ -9711,6 +10843,12 @@
         <v>0</v>
       </c>
       <c r="M189" t="n">
+        <v>0</v>
+      </c>
+      <c r="N189" t="n">
+        <v>0</v>
+      </c>
+      <c r="O189" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9760,6 +10898,12 @@
         <v>0</v>
       </c>
       <c r="M190" t="n">
+        <v>0</v>
+      </c>
+      <c r="N190" t="n">
+        <v>0</v>
+      </c>
+      <c r="O190" t="n">
         <v>32</v>
       </c>
     </row>
@@ -9809,6 +10953,12 @@
         <v>0</v>
       </c>
       <c r="M191" t="n">
+        <v>0</v>
+      </c>
+      <c r="N191" t="n">
+        <v>0</v>
+      </c>
+      <c r="O191" t="n">
         <v>13</v>
       </c>
     </row>
@@ -9858,6 +11008,12 @@
         <v>0</v>
       </c>
       <c r="M192" t="n">
+        <v>0</v>
+      </c>
+      <c r="N192" t="n">
+        <v>0</v>
+      </c>
+      <c r="O192" t="n">
         <v>9</v>
       </c>
     </row>
@@ -9909,6 +11065,12 @@
       <c r="M193" t="n">
         <v>0</v>
       </c>
+      <c r="N193" t="n">
+        <v>0</v>
+      </c>
+      <c r="O193" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="n">
@@ -9956,6 +11118,12 @@
         <v>0</v>
       </c>
       <c r="M194" t="n">
+        <v>0</v>
+      </c>
+      <c r="N194" t="n">
+        <v>0</v>
+      </c>
+      <c r="O194" t="n">
         <v>1</v>
       </c>
     </row>
@@ -10007,6 +11175,12 @@
       <c r="M195" t="n">
         <v>0</v>
       </c>
+      <c r="N195" t="n">
+        <v>0</v>
+      </c>
+      <c r="O195" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="n">
@@ -10056,6 +11230,12 @@
       <c r="M196" t="n">
         <v>0</v>
       </c>
+      <c r="N196" t="n">
+        <v>0</v>
+      </c>
+      <c r="O196" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="n">
@@ -10105,6 +11285,12 @@
       <c r="M197" t="n">
         <v>0</v>
       </c>
+      <c r="N197" t="n">
+        <v>0</v>
+      </c>
+      <c r="O197" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="n">
@@ -10152,6 +11338,12 @@
         <v>0</v>
       </c>
       <c r="M198" t="n">
+        <v>0</v>
+      </c>
+      <c r="N198" t="n">
+        <v>0</v>
+      </c>
+      <c r="O198" t="n">
         <v>39</v>
       </c>
     </row>
@@ -10201,6 +11393,12 @@
         <v>0</v>
       </c>
       <c r="M199" t="n">
+        <v>0</v>
+      </c>
+      <c r="N199" t="n">
+        <v>0</v>
+      </c>
+      <c r="O199" t="n">
         <v>10</v>
       </c>
     </row>
@@ -10250,6 +11448,12 @@
         <v>0</v>
       </c>
       <c r="M200" t="n">
+        <v>0</v>
+      </c>
+      <c r="N200" t="n">
+        <v>0</v>
+      </c>
+      <c r="O200" t="n">
         <v>81</v>
       </c>
     </row>
@@ -10299,11 +11503,17 @@
         <v>0</v>
       </c>
       <c r="M201" t="n">
+        <v>0</v>
+      </c>
+      <c r="N201" t="n">
+        <v>0</v>
+      </c>
+      <c r="O201" t="n">
         <v>3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M201"/>
+  <autoFilter ref="A1:O201"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update 12/10/2026 (BC 0757 report, 10-12-GAF2)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gate-move-summary.xlsx
+++ b/docs/gate-move-summary.xlsx
@@ -11879,7 +11879,7 @@
         <v>1</v>
       </c>
       <c r="J208" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K208" t="n">
         <v>0</v>
@@ -11894,7 +11894,7 @@
         <v>0</v>
       </c>
       <c r="O208" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="209">
@@ -11922,7 +11922,7 @@
         </is>
       </c>
       <c r="F209" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G209" t="n">
         <v>0</v>
@@ -11934,7 +11934,7 @@
         <v>0</v>
       </c>
       <c r="J209" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K209" t="n">
         <v>0</v>
@@ -11949,7 +11949,7 @@
         <v>0</v>
       </c>
       <c r="O209" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="210">
@@ -15671,10 +15671,10 @@
         </is>
       </c>
       <c r="E105" t="n">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="F105" t="n">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="G105" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Combine all system files of a day; accept blank Location header; update 15/10 (PW FINAL + ADDINF)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gate-move-summary.xlsx
+++ b/docs/gate-move-summary.xlsx
@@ -14672,7 +14672,7 @@
         </is>
       </c>
       <c r="F259" t="n">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="G259" t="n">
         <v>0</v>
@@ -14699,7 +14699,7 @@
         <v>0</v>
       </c>
       <c r="O259" t="n">
-        <v>57</v>
+        <v>67</v>
       </c>
     </row>
     <row r="260">
@@ -18596,10 +18596,10 @@
         </is>
       </c>
       <c r="E130" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="F130" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G130" t="n">
         <v>0</v>
@@ -18628,10 +18628,10 @@
         <v>105</v>
       </c>
       <c r="F131" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G131" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update 15/10/2026 (10-15-gate): all match
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gate-move-summary.xlsx
+++ b/docs/gate-move-summary.xlsx
@@ -18454,10 +18454,10 @@
         <v>58</v>
       </c>
       <c r="F125" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="G125" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="126">
@@ -18483,10 +18483,10 @@
         <v>47</v>
       </c>
       <c r="F126" t="n">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="G126" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="127">

</xml_diff>

<commit_message>
Combined system files: dedupe counted moves by direction (code may change OEV->OEP)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gate-move-summary.xlsx
+++ b/docs/gate-move-summary.xlsx
@@ -18454,10 +18454,10 @@
         <v>58</v>
       </c>
       <c r="F125" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G125" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="126">

</xml_diff>

<commit_message>
Update 17/10/2026 (CELLO FINAL, BC 0807, 10-17-GAF): all match
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gate-move-summary.xlsx
+++ b/docs/gate-move-summary.xlsx
@@ -16163,13 +16163,13 @@
         <v>0</v>
       </c>
       <c r="H286" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I286" t="n">
         <v>1</v>
       </c>
       <c r="J286" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K286" t="n">
         <v>0</v>
@@ -16212,7 +16212,7 @@
         </is>
       </c>
       <c r="F287" t="n">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="G287" t="n">
         <v>0</v>
@@ -16239,7 +16239,7 @@
         <v>0</v>
       </c>
       <c r="O287" t="n">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="288">
@@ -16273,7 +16273,7 @@
         <v>0</v>
       </c>
       <c r="H288" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I288" t="n">
         <v>0</v>
@@ -16294,7 +16294,7 @@
         <v>0</v>
       </c>
       <c r="O288" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="289">
@@ -16658,7 +16658,7 @@
         <v>0</v>
       </c>
       <c r="H295" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I295" t="n">
         <v>0</v>
@@ -16679,7 +16679,7 @@
         <v>0</v>
       </c>
       <c r="O295" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="296">
@@ -21202,10 +21202,10 @@
         </is>
       </c>
       <c r="E144" t="n">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="F144" t="n">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="G144" t="n">
         <v>0</v>
@@ -21231,10 +21231,10 @@
         </is>
       </c>
       <c r="E145" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F145" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G145" t="n">
         <v>0</v>
@@ -21318,13 +21318,13 @@
         </is>
       </c>
       <c r="E148" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="F148" t="n">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="G148" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="149">

</xml_diff>

<commit_message>
Update 19/10/2026 (10-19-GAF): all match
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gate-move-summary.xlsx
+++ b/docs/gate-move-summary.xlsx
@@ -22595,10 +22595,10 @@
         <v>83</v>
       </c>
       <c r="F154" t="n">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="G154" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="155">
@@ -22624,10 +22624,10 @@
         <v>175</v>
       </c>
       <c r="F155" t="n">
-        <v>156</v>
+        <v>175</v>
       </c>
       <c r="G155" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
     </row>
     <row r="156">

</xml_diff>

<commit_message>
System file detection: skip date-range work files, require one-day exports; update 20/10/2026
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gate-move-summary.xlsx
+++ b/docs/gate-move-summary.xlsx
@@ -18137,13 +18137,13 @@
         </is>
       </c>
       <c r="F322" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G322" t="n">
         <v>0</v>
       </c>
       <c r="H322" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="I322" t="n">
         <v>0</v>
@@ -18164,7 +18164,7 @@
         <v>0</v>
       </c>
       <c r="O322" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="323">
@@ -18247,7 +18247,7 @@
         </is>
       </c>
       <c r="F324" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G324" t="n">
         <v>0</v>
@@ -18274,7 +18274,7 @@
         <v>0</v>
       </c>
       <c r="O324" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="325">
@@ -23924,10 +23924,10 @@
         </is>
       </c>
       <c r="E162" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F162" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G162" t="n">
         <v>0</v>
@@ -23953,10 +23953,10 @@
         </is>
       </c>
       <c r="E163" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F163" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G163" t="n">
         <v>0</v>
@@ -24014,10 +24014,10 @@
         <v>116</v>
       </c>
       <c r="F165" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G165" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="166">

</xml_diff>

<commit_message>
Update 20/10/2026 (BC 0803): all match
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gate-move-summary.xlsx
+++ b/docs/gate-move-summary.xlsx
@@ -18470,7 +18470,7 @@
         <v>66</v>
       </c>
       <c r="G328" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H328" t="n">
         <v>32</v>
@@ -18494,7 +18494,7 @@
         <v>0</v>
       </c>
       <c r="O328" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="329">
@@ -24011,13 +24011,13 @@
         </is>
       </c>
       <c r="E165" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F165" t="n">
         <v>117</v>
       </c>
       <c r="G165" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="166">

</xml_diff>

<commit_message>
MISSING BL No: ignore notes typed in BKG#/BOOKING IN; add 21/10/2026
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gate-move-summary.xlsx
+++ b/docs/gate-move-summary.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Compare" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daily Summary'!$A$1:$O$341</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'System Compare'!$A$1:$G$171</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daily Summary'!$A$1:$O$361</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'System Compare'!$A$1:$G$181</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O341"/>
+  <dimension ref="A1:O361"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19212,8 +19212,1108 @@
         <v>0</v>
       </c>
     </row>
+    <row r="342">
+      <c r="A342" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>SMART BKK</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>BKK25</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>Consignee</t>
+        </is>
+      </c>
+      <c r="F342" t="n">
+        <v>13</v>
+      </c>
+      <c r="G342" t="n">
+        <v>0</v>
+      </c>
+      <c r="H342" t="n">
+        <v>3</v>
+      </c>
+      <c r="I342" t="n">
+        <v>0</v>
+      </c>
+      <c r="J342" t="n">
+        <v>0</v>
+      </c>
+      <c r="K342" t="n">
+        <v>0</v>
+      </c>
+      <c r="L342" t="n">
+        <v>0</v>
+      </c>
+      <c r="M342" t="n">
+        <v>0</v>
+      </c>
+      <c r="N342" t="n">
+        <v>0</v>
+      </c>
+      <c r="O342" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>SMART BKK</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>BKK25</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F343" t="n">
+        <v>0</v>
+      </c>
+      <c r="G343" t="n">
+        <v>0</v>
+      </c>
+      <c r="H343" t="n">
+        <v>0</v>
+      </c>
+      <c r="I343" t="n">
+        <v>0</v>
+      </c>
+      <c r="J343" t="n">
+        <v>0</v>
+      </c>
+      <c r="K343" t="n">
+        <v>0</v>
+      </c>
+      <c r="L343" t="n">
+        <v>0</v>
+      </c>
+      <c r="M343" t="n">
+        <v>0</v>
+      </c>
+      <c r="N343" t="n">
+        <v>0</v>
+      </c>
+      <c r="O343" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>SMART BKK</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>BKK25</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>Shipper</t>
+        </is>
+      </c>
+      <c r="F344" t="n">
+        <v>5</v>
+      </c>
+      <c r="G344" t="n">
+        <v>0</v>
+      </c>
+      <c r="H344" t="n">
+        <v>3</v>
+      </c>
+      <c r="I344" t="n">
+        <v>0</v>
+      </c>
+      <c r="J344" t="n">
+        <v>0</v>
+      </c>
+      <c r="K344" t="n">
+        <v>0</v>
+      </c>
+      <c r="L344" t="n">
+        <v>0</v>
+      </c>
+      <c r="M344" t="n">
+        <v>0</v>
+      </c>
+      <c r="N344" t="n">
+        <v>0</v>
+      </c>
+      <c r="O344" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>SMART BKK</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>BKK25</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F345" t="n">
+        <v>0</v>
+      </c>
+      <c r="G345" t="n">
+        <v>0</v>
+      </c>
+      <c r="H345" t="n">
+        <v>0</v>
+      </c>
+      <c r="I345" t="n">
+        <v>0</v>
+      </c>
+      <c r="J345" t="n">
+        <v>0</v>
+      </c>
+      <c r="K345" t="n">
+        <v>0</v>
+      </c>
+      <c r="L345" t="n">
+        <v>0</v>
+      </c>
+      <c r="M345" t="n">
+        <v>0</v>
+      </c>
+      <c r="N345" t="n">
+        <v>0</v>
+      </c>
+      <c r="O345" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>BKK27</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>Consignee</t>
+        </is>
+      </c>
+      <c r="F346" t="n">
+        <v>14</v>
+      </c>
+      <c r="G346" t="n">
+        <v>0</v>
+      </c>
+      <c r="H346" t="n">
+        <v>26</v>
+      </c>
+      <c r="I346" t="n">
+        <v>1</v>
+      </c>
+      <c r="J346" t="n">
+        <v>4</v>
+      </c>
+      <c r="K346" t="n">
+        <v>0</v>
+      </c>
+      <c r="L346" t="n">
+        <v>0</v>
+      </c>
+      <c r="M346" t="n">
+        <v>0</v>
+      </c>
+      <c r="N346" t="n">
+        <v>0</v>
+      </c>
+      <c r="O346" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>BKK27</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F347" t="n">
+        <v>12</v>
+      </c>
+      <c r="G347" t="n">
+        <v>0</v>
+      </c>
+      <c r="H347" t="n">
+        <v>0</v>
+      </c>
+      <c r="I347" t="n">
+        <v>0</v>
+      </c>
+      <c r="J347" t="n">
+        <v>0</v>
+      </c>
+      <c r="K347" t="n">
+        <v>0</v>
+      </c>
+      <c r="L347" t="n">
+        <v>0</v>
+      </c>
+      <c r="M347" t="n">
+        <v>0</v>
+      </c>
+      <c r="N347" t="n">
+        <v>0</v>
+      </c>
+      <c r="O347" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>BKK27</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>Shipper</t>
+        </is>
+      </c>
+      <c r="F348" t="n">
+        <v>38</v>
+      </c>
+      <c r="G348" t="n">
+        <v>0</v>
+      </c>
+      <c r="H348" t="n">
+        <v>32</v>
+      </c>
+      <c r="I348" t="n">
+        <v>1</v>
+      </c>
+      <c r="J348" t="n">
+        <v>7</v>
+      </c>
+      <c r="K348" t="n">
+        <v>0</v>
+      </c>
+      <c r="L348" t="n">
+        <v>0</v>
+      </c>
+      <c r="M348" t="n">
+        <v>0</v>
+      </c>
+      <c r="N348" t="n">
+        <v>0</v>
+      </c>
+      <c r="O348" t="n">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>BKK27</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F349" t="n">
+        <v>0</v>
+      </c>
+      <c r="G349" t="n">
+        <v>0</v>
+      </c>
+      <c r="H349" t="n">
+        <v>0</v>
+      </c>
+      <c r="I349" t="n">
+        <v>0</v>
+      </c>
+      <c r="J349" t="n">
+        <v>2</v>
+      </c>
+      <c r="K349" t="n">
+        <v>0</v>
+      </c>
+      <c r="L349" t="n">
+        <v>0</v>
+      </c>
+      <c r="M349" t="n">
+        <v>0</v>
+      </c>
+      <c r="N349" t="n">
+        <v>0</v>
+      </c>
+      <c r="O349" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>HAST</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>LCH27</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>Consignee</t>
+        </is>
+      </c>
+      <c r="F350" t="n">
+        <v>8</v>
+      </c>
+      <c r="G350" t="n">
+        <v>0</v>
+      </c>
+      <c r="H350" t="n">
+        <v>5</v>
+      </c>
+      <c r="I350" t="n">
+        <v>0</v>
+      </c>
+      <c r="J350" t="n">
+        <v>1</v>
+      </c>
+      <c r="K350" t="n">
+        <v>0</v>
+      </c>
+      <c r="L350" t="n">
+        <v>0</v>
+      </c>
+      <c r="M350" t="n">
+        <v>0</v>
+      </c>
+      <c r="N350" t="n">
+        <v>0</v>
+      </c>
+      <c r="O350" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>HAST</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>LCH27</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F351" t="n">
+        <v>0</v>
+      </c>
+      <c r="G351" t="n">
+        <v>0</v>
+      </c>
+      <c r="H351" t="n">
+        <v>1</v>
+      </c>
+      <c r="I351" t="n">
+        <v>0</v>
+      </c>
+      <c r="J351" t="n">
+        <v>0</v>
+      </c>
+      <c r="K351" t="n">
+        <v>0</v>
+      </c>
+      <c r="L351" t="n">
+        <v>0</v>
+      </c>
+      <c r="M351" t="n">
+        <v>0</v>
+      </c>
+      <c r="N351" t="n">
+        <v>0</v>
+      </c>
+      <c r="O351" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>HAST</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>LCH27</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>Shipper</t>
+        </is>
+      </c>
+      <c r="F352" t="n">
+        <v>27</v>
+      </c>
+      <c r="G352" t="n">
+        <v>0</v>
+      </c>
+      <c r="H352" t="n">
+        <v>7</v>
+      </c>
+      <c r="I352" t="n">
+        <v>0</v>
+      </c>
+      <c r="J352" t="n">
+        <v>3</v>
+      </c>
+      <c r="K352" t="n">
+        <v>0</v>
+      </c>
+      <c r="L352" t="n">
+        <v>0</v>
+      </c>
+      <c r="M352" t="n">
+        <v>0</v>
+      </c>
+      <c r="N352" t="n">
+        <v>0</v>
+      </c>
+      <c r="O352" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>HAST</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>LCH27</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F353" t="n">
+        <v>0</v>
+      </c>
+      <c r="G353" t="n">
+        <v>0</v>
+      </c>
+      <c r="H353" t="n">
+        <v>0</v>
+      </c>
+      <c r="I353" t="n">
+        <v>0</v>
+      </c>
+      <c r="J353" t="n">
+        <v>0</v>
+      </c>
+      <c r="K353" t="n">
+        <v>0</v>
+      </c>
+      <c r="L353" t="n">
+        <v>0</v>
+      </c>
+      <c r="M353" t="n">
+        <v>0</v>
+      </c>
+      <c r="N353" t="n">
+        <v>0</v>
+      </c>
+      <c r="O353" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>LCH28</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>Consignee</t>
+        </is>
+      </c>
+      <c r="F354" t="n">
+        <v>0</v>
+      </c>
+      <c r="G354" t="n">
+        <v>0</v>
+      </c>
+      <c r="H354" t="n">
+        <v>2</v>
+      </c>
+      <c r="I354" t="n">
+        <v>0</v>
+      </c>
+      <c r="J354" t="n">
+        <v>0</v>
+      </c>
+      <c r="K354" t="n">
+        <v>0</v>
+      </c>
+      <c r="L354" t="n">
+        <v>0</v>
+      </c>
+      <c r="M354" t="n">
+        <v>0</v>
+      </c>
+      <c r="N354" t="n">
+        <v>0</v>
+      </c>
+      <c r="O354" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>LCH28</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F355" t="n">
+        <v>0</v>
+      </c>
+      <c r="G355" t="n">
+        <v>0</v>
+      </c>
+      <c r="H355" t="n">
+        <v>6</v>
+      </c>
+      <c r="I355" t="n">
+        <v>0</v>
+      </c>
+      <c r="J355" t="n">
+        <v>0</v>
+      </c>
+      <c r="K355" t="n">
+        <v>0</v>
+      </c>
+      <c r="L355" t="n">
+        <v>0</v>
+      </c>
+      <c r="M355" t="n">
+        <v>0</v>
+      </c>
+      <c r="N355" t="n">
+        <v>0</v>
+      </c>
+      <c r="O355" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>LCH28</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>Shipper</t>
+        </is>
+      </c>
+      <c r="F356" t="n">
+        <v>0</v>
+      </c>
+      <c r="G356" t="n">
+        <v>0</v>
+      </c>
+      <c r="H356" t="n">
+        <v>4</v>
+      </c>
+      <c r="I356" t="n">
+        <v>0</v>
+      </c>
+      <c r="J356" t="n">
+        <v>0</v>
+      </c>
+      <c r="K356" t="n">
+        <v>0</v>
+      </c>
+      <c r="L356" t="n">
+        <v>0</v>
+      </c>
+      <c r="M356" t="n">
+        <v>0</v>
+      </c>
+      <c r="N356" t="n">
+        <v>0</v>
+      </c>
+      <c r="O356" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>LCH28</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F357" t="n">
+        <v>0</v>
+      </c>
+      <c r="G357" t="n">
+        <v>0</v>
+      </c>
+      <c r="H357" t="n">
+        <v>0</v>
+      </c>
+      <c r="I357" t="n">
+        <v>0</v>
+      </c>
+      <c r="J357" t="n">
+        <v>0</v>
+      </c>
+      <c r="K357" t="n">
+        <v>0</v>
+      </c>
+      <c r="L357" t="n">
+        <v>0</v>
+      </c>
+      <c r="M357" t="n">
+        <v>0</v>
+      </c>
+      <c r="N357" t="n">
+        <v>0</v>
+      </c>
+      <c r="O357" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>Consignee</t>
+        </is>
+      </c>
+      <c r="F358" t="n">
+        <v>5</v>
+      </c>
+      <c r="G358" t="n">
+        <v>0</v>
+      </c>
+      <c r="H358" t="n">
+        <v>8</v>
+      </c>
+      <c r="I358" t="n">
+        <v>0</v>
+      </c>
+      <c r="J358" t="n">
+        <v>0</v>
+      </c>
+      <c r="K358" t="n">
+        <v>0</v>
+      </c>
+      <c r="L358" t="n">
+        <v>0</v>
+      </c>
+      <c r="M358" t="n">
+        <v>0</v>
+      </c>
+      <c r="N358" t="n">
+        <v>0</v>
+      </c>
+      <c r="O358" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F359" t="n">
+        <v>0</v>
+      </c>
+      <c r="G359" t="n">
+        <v>0</v>
+      </c>
+      <c r="H359" t="n">
+        <v>0</v>
+      </c>
+      <c r="I359" t="n">
+        <v>0</v>
+      </c>
+      <c r="J359" t="n">
+        <v>0</v>
+      </c>
+      <c r="K359" t="n">
+        <v>0</v>
+      </c>
+      <c r="L359" t="n">
+        <v>0</v>
+      </c>
+      <c r="M359" t="n">
+        <v>0</v>
+      </c>
+      <c r="N359" t="n">
+        <v>0</v>
+      </c>
+      <c r="O359" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>Shipper</t>
+        </is>
+      </c>
+      <c r="F360" t="n">
+        <v>74</v>
+      </c>
+      <c r="G360" t="n">
+        <v>0</v>
+      </c>
+      <c r="H360" t="n">
+        <v>79</v>
+      </c>
+      <c r="I360" t="n">
+        <v>0</v>
+      </c>
+      <c r="J360" t="n">
+        <v>0</v>
+      </c>
+      <c r="K360" t="n">
+        <v>0</v>
+      </c>
+      <c r="L360" t="n">
+        <v>0</v>
+      </c>
+      <c r="M360" t="n">
+        <v>0</v>
+      </c>
+      <c r="N360" t="n">
+        <v>0</v>
+      </c>
+      <c r="O360" t="n">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F361" t="n">
+        <v>4</v>
+      </c>
+      <c r="G361" t="n">
+        <v>0</v>
+      </c>
+      <c r="H361" t="n">
+        <v>3</v>
+      </c>
+      <c r="I361" t="n">
+        <v>0</v>
+      </c>
+      <c r="J361" t="n">
+        <v>0</v>
+      </c>
+      <c r="K361" t="n">
+        <v>0</v>
+      </c>
+      <c r="L361" t="n">
+        <v>0</v>
+      </c>
+      <c r="M361" t="n">
+        <v>0</v>
+      </c>
+      <c r="N361" t="n">
+        <v>0</v>
+      </c>
+      <c r="O361" t="n">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O341"/>
+  <autoFilter ref="A1:O361"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -19224,7 +20324,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G171"/>
+  <dimension ref="A1:G181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24194,8 +25294,298 @@
         <v>0</v>
       </c>
     </row>
+    <row r="172">
+      <c r="A172" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>SMART BKK</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>BKK25</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E172" t="n">
+        <v>16</v>
+      </c>
+      <c r="F172" t="n">
+        <v>16</v>
+      </c>
+      <c r="G172" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>SMART BKK</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>BKK25</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E173" t="n">
+        <v>8</v>
+      </c>
+      <c r="F173" t="n">
+        <v>7</v>
+      </c>
+      <c r="G173" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>BKK27</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E174" t="n">
+        <v>57</v>
+      </c>
+      <c r="F174" t="n">
+        <v>57</v>
+      </c>
+      <c r="G174" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>BKK27</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E175" t="n">
+        <v>80</v>
+      </c>
+      <c r="F175" t="n">
+        <v>80</v>
+      </c>
+      <c r="G175" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>HAST</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>LCH27</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E176" t="n">
+        <v>15</v>
+      </c>
+      <c r="F176" t="n">
+        <v>14</v>
+      </c>
+      <c r="G176" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>HAST</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>LCH27</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E177" t="n">
+        <v>37</v>
+      </c>
+      <c r="F177" t="n">
+        <v>37</v>
+      </c>
+      <c r="G177" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>LCH28</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E178" t="n">
+        <v>8</v>
+      </c>
+      <c r="F178" t="n">
+        <v>1</v>
+      </c>
+      <c r="G178" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>LCH28</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E179" t="n">
+        <v>4</v>
+      </c>
+      <c r="F179" t="n">
+        <v>5</v>
+      </c>
+      <c r="G179" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E180" t="n">
+        <v>13</v>
+      </c>
+      <c r="F180" t="n">
+        <v>13</v>
+      </c>
+      <c r="G180" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E181" t="n">
+        <v>160</v>
+      </c>
+      <c r="F181" t="n">
+        <v>160</v>
+      </c>
+      <c r="G181" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G171"/>
+  <autoFilter ref="A1:G181"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update 21/10/2026 (BC 0758, 10-21-GAFF)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gate-move-summary.xlsx
+++ b/docs/gate-move-summary.xlsx
@@ -19573,7 +19573,7 @@
         <v>0</v>
       </c>
       <c r="H348" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I348" t="n">
         <v>1</v>
@@ -19594,7 +19594,7 @@
         <v>0</v>
       </c>
       <c r="O348" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="349">
@@ -19622,13 +19622,13 @@
         </is>
       </c>
       <c r="F349" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G349" t="n">
         <v>0</v>
       </c>
       <c r="H349" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I349" t="n">
         <v>0</v>
@@ -19649,7 +19649,7 @@
         <v>0</v>
       </c>
       <c r="O349" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="350">
@@ -25401,13 +25401,13 @@
         </is>
       </c>
       <c r="E175" t="n">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="F175" t="n">
         <v>80</v>
       </c>
       <c r="G175" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="176">

</xml_diff>

<commit_message>
Also check next-day-named system exports; update 21/10/2026 (10-22-GAGA)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gate-move-summary.xlsx
+++ b/docs/gate-move-summary.xlsx
@@ -25404,10 +25404,10 @@
         <v>86</v>
       </c>
       <c r="F175" t="n">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G175" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="176">

</xml_diff>

<commit_message>
Update 21/10/2026 (CELLO FINAL): all match
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gate-move-summary.xlsx
+++ b/docs/gate-move-summary.xlsx
@@ -19903,7 +19903,7 @@
         <v>0</v>
       </c>
       <c r="H354" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I354" t="n">
         <v>0</v>
@@ -19924,7 +19924,7 @@
         <v>0</v>
       </c>
       <c r="O354" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="355">
@@ -19958,7 +19958,7 @@
         <v>0</v>
       </c>
       <c r="H355" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I355" t="n">
         <v>0</v>
@@ -19979,7 +19979,7 @@
         <v>0</v>
       </c>
       <c r="O355" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="356">
@@ -20013,7 +20013,7 @@
         <v>0</v>
       </c>
       <c r="H356" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I356" t="n">
         <v>0</v>
@@ -20034,7 +20034,7 @@
         <v>0</v>
       </c>
       <c r="O356" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="357">
@@ -25517,13 +25517,13 @@
         </is>
       </c>
       <c r="E179" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F179" t="n">
         <v>5</v>
       </c>
       <c r="G179" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="180">

</xml_diff>

<commit_message>
22/10/2026: 3 PW containers keyed into the system (10-22-KEYED)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gate-move-summary.xlsx
+++ b/docs/gate-move-summary.xlsx
@@ -26968,10 +26968,10 @@
         <v>89</v>
       </c>
       <c r="F191" t="n">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="G191" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update 22/10/2026 (BC 0807, SMART, 10-22-GAF2): all match
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gate-move-summary.xlsx
+++ b/docs/gate-move-summary.xlsx
@@ -20343,7 +20343,7 @@
         <v>0</v>
       </c>
       <c r="H362" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I362" t="n">
         <v>0</v>
@@ -20364,7 +20364,7 @@
         <v>0</v>
       </c>
       <c r="O362" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="363">
@@ -20722,7 +20722,7 @@
         </is>
       </c>
       <c r="F369" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G369" t="n">
         <v>0</v>
@@ -20749,7 +20749,7 @@
         <v>0</v>
       </c>
       <c r="O369" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="370">
@@ -26704,10 +26704,10 @@
         </is>
       </c>
       <c r="E182" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F182" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G182" t="n">
         <v>0</v>
@@ -26791,10 +26791,10 @@
         </is>
       </c>
       <c r="E185" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="F185" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="G185" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Add 24/10/2026 (SMART, BC, PW open; HAST, CELLO closed)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gate-move-summary.xlsx
+++ b/docs/gate-move-summary.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Compare" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daily Summary'!$A$1:$O$381</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'System Compare'!$A$1:$G$191</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daily Summary'!$A$1:$O$393</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'System Compare'!$A$1:$G$197</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O381"/>
+  <dimension ref="A1:O393"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21412,8 +21412,668 @@
         <v>7</v>
       </c>
     </row>
+    <row r="382">
+      <c r="A382" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>SMART BKK</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>BKK25</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>Consignee</t>
+        </is>
+      </c>
+      <c r="F382" t="n">
+        <v>7</v>
+      </c>
+      <c r="G382" t="n">
+        <v>0</v>
+      </c>
+      <c r="H382" t="n">
+        <v>8</v>
+      </c>
+      <c r="I382" t="n">
+        <v>0</v>
+      </c>
+      <c r="J382" t="n">
+        <v>0</v>
+      </c>
+      <c r="K382" t="n">
+        <v>0</v>
+      </c>
+      <c r="L382" t="n">
+        <v>0</v>
+      </c>
+      <c r="M382" t="n">
+        <v>0</v>
+      </c>
+      <c r="N382" t="n">
+        <v>0</v>
+      </c>
+      <c r="O382" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>SMART BKK</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>BKK25</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F383" t="n">
+        <v>0</v>
+      </c>
+      <c r="G383" t="n">
+        <v>0</v>
+      </c>
+      <c r="H383" t="n">
+        <v>0</v>
+      </c>
+      <c r="I383" t="n">
+        <v>0</v>
+      </c>
+      <c r="J383" t="n">
+        <v>0</v>
+      </c>
+      <c r="K383" t="n">
+        <v>0</v>
+      </c>
+      <c r="L383" t="n">
+        <v>0</v>
+      </c>
+      <c r="M383" t="n">
+        <v>0</v>
+      </c>
+      <c r="N383" t="n">
+        <v>0</v>
+      </c>
+      <c r="O383" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>SMART BKK</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>BKK25</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>Shipper</t>
+        </is>
+      </c>
+      <c r="F384" t="n">
+        <v>5</v>
+      </c>
+      <c r="G384" t="n">
+        <v>0</v>
+      </c>
+      <c r="H384" t="n">
+        <v>0</v>
+      </c>
+      <c r="I384" t="n">
+        <v>0</v>
+      </c>
+      <c r="J384" t="n">
+        <v>0</v>
+      </c>
+      <c r="K384" t="n">
+        <v>0</v>
+      </c>
+      <c r="L384" t="n">
+        <v>0</v>
+      </c>
+      <c r="M384" t="n">
+        <v>0</v>
+      </c>
+      <c r="N384" t="n">
+        <v>0</v>
+      </c>
+      <c r="O384" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>SMART BKK</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>BKK25</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F385" t="n">
+        <v>2</v>
+      </c>
+      <c r="G385" t="n">
+        <v>0</v>
+      </c>
+      <c r="H385" t="n">
+        <v>0</v>
+      </c>
+      <c r="I385" t="n">
+        <v>0</v>
+      </c>
+      <c r="J385" t="n">
+        <v>0</v>
+      </c>
+      <c r="K385" t="n">
+        <v>0</v>
+      </c>
+      <c r="L385" t="n">
+        <v>0</v>
+      </c>
+      <c r="M385" t="n">
+        <v>0</v>
+      </c>
+      <c r="N385" t="n">
+        <v>0</v>
+      </c>
+      <c r="O385" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>BKK27</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>Consignee</t>
+        </is>
+      </c>
+      <c r="F386" t="n">
+        <v>14</v>
+      </c>
+      <c r="G386" t="n">
+        <v>0</v>
+      </c>
+      <c r="H386" t="n">
+        <v>33</v>
+      </c>
+      <c r="I386" t="n">
+        <v>0</v>
+      </c>
+      <c r="J386" t="n">
+        <v>3</v>
+      </c>
+      <c r="K386" t="n">
+        <v>0</v>
+      </c>
+      <c r="L386" t="n">
+        <v>0</v>
+      </c>
+      <c r="M386" t="n">
+        <v>0</v>
+      </c>
+      <c r="N386" t="n">
+        <v>0</v>
+      </c>
+      <c r="O386" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>BKK27</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F387" t="n">
+        <v>0</v>
+      </c>
+      <c r="G387" t="n">
+        <v>0</v>
+      </c>
+      <c r="H387" t="n">
+        <v>0</v>
+      </c>
+      <c r="I387" t="n">
+        <v>0</v>
+      </c>
+      <c r="J387" t="n">
+        <v>0</v>
+      </c>
+      <c r="K387" t="n">
+        <v>0</v>
+      </c>
+      <c r="L387" t="n">
+        <v>0</v>
+      </c>
+      <c r="M387" t="n">
+        <v>0</v>
+      </c>
+      <c r="N387" t="n">
+        <v>0</v>
+      </c>
+      <c r="O387" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>BKK27</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>Shipper</t>
+        </is>
+      </c>
+      <c r="F388" t="n">
+        <v>27</v>
+      </c>
+      <c r="G388" t="n">
+        <v>0</v>
+      </c>
+      <c r="H388" t="n">
+        <v>13</v>
+      </c>
+      <c r="I388" t="n">
+        <v>1</v>
+      </c>
+      <c r="J388" t="n">
+        <v>3</v>
+      </c>
+      <c r="K388" t="n">
+        <v>0</v>
+      </c>
+      <c r="L388" t="n">
+        <v>0</v>
+      </c>
+      <c r="M388" t="n">
+        <v>0</v>
+      </c>
+      <c r="N388" t="n">
+        <v>0</v>
+      </c>
+      <c r="O388" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>BKK27</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F389" t="n">
+        <v>0</v>
+      </c>
+      <c r="G389" t="n">
+        <v>0</v>
+      </c>
+      <c r="H389" t="n">
+        <v>0</v>
+      </c>
+      <c r="I389" t="n">
+        <v>0</v>
+      </c>
+      <c r="J389" t="n">
+        <v>1</v>
+      </c>
+      <c r="K389" t="n">
+        <v>0</v>
+      </c>
+      <c r="L389" t="n">
+        <v>0</v>
+      </c>
+      <c r="M389" t="n">
+        <v>0</v>
+      </c>
+      <c r="N389" t="n">
+        <v>0</v>
+      </c>
+      <c r="O389" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>Consignee</t>
+        </is>
+      </c>
+      <c r="F390" t="n">
+        <v>16</v>
+      </c>
+      <c r="G390" t="n">
+        <v>0</v>
+      </c>
+      <c r="H390" t="n">
+        <v>18</v>
+      </c>
+      <c r="I390" t="n">
+        <v>0</v>
+      </c>
+      <c r="J390" t="n">
+        <v>0</v>
+      </c>
+      <c r="K390" t="n">
+        <v>0</v>
+      </c>
+      <c r="L390" t="n">
+        <v>0</v>
+      </c>
+      <c r="M390" t="n">
+        <v>0</v>
+      </c>
+      <c r="N390" t="n">
+        <v>0</v>
+      </c>
+      <c r="O390" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F391" t="n">
+        <v>0</v>
+      </c>
+      <c r="G391" t="n">
+        <v>0</v>
+      </c>
+      <c r="H391" t="n">
+        <v>1</v>
+      </c>
+      <c r="I391" t="n">
+        <v>0</v>
+      </c>
+      <c r="J391" t="n">
+        <v>0</v>
+      </c>
+      <c r="K391" t="n">
+        <v>0</v>
+      </c>
+      <c r="L391" t="n">
+        <v>0</v>
+      </c>
+      <c r="M391" t="n">
+        <v>0</v>
+      </c>
+      <c r="N391" t="n">
+        <v>0</v>
+      </c>
+      <c r="O391" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>Shipper</t>
+        </is>
+      </c>
+      <c r="F392" t="n">
+        <v>21</v>
+      </c>
+      <c r="G392" t="n">
+        <v>0</v>
+      </c>
+      <c r="H392" t="n">
+        <v>26</v>
+      </c>
+      <c r="I392" t="n">
+        <v>0</v>
+      </c>
+      <c r="J392" t="n">
+        <v>0</v>
+      </c>
+      <c r="K392" t="n">
+        <v>0</v>
+      </c>
+      <c r="L392" t="n">
+        <v>0</v>
+      </c>
+      <c r="M392" t="n">
+        <v>0</v>
+      </c>
+      <c r="N392" t="n">
+        <v>0</v>
+      </c>
+      <c r="O392" t="n">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="F393" t="n">
+        <v>3</v>
+      </c>
+      <c r="G393" t="n">
+        <v>0</v>
+      </c>
+      <c r="H393" t="n">
+        <v>1</v>
+      </c>
+      <c r="I393" t="n">
+        <v>0</v>
+      </c>
+      <c r="J393" t="n">
+        <v>0</v>
+      </c>
+      <c r="K393" t="n">
+        <v>0</v>
+      </c>
+      <c r="L393" t="n">
+        <v>0</v>
+      </c>
+      <c r="M393" t="n">
+        <v>0</v>
+      </c>
+      <c r="N393" t="n">
+        <v>0</v>
+      </c>
+      <c r="O393" t="n">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O381"/>
+  <autoFilter ref="A1:O393"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -21424,7 +22084,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G191"/>
+  <dimension ref="A1:G197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26974,8 +27634,182 @@
         <v>0</v>
       </c>
     </row>
+    <row r="192">
+      <c r="A192" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>SMART BKK</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>BKK25</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E192" t="n">
+        <v>15</v>
+      </c>
+      <c r="F192" t="n">
+        <v>15</v>
+      </c>
+      <c r="G192" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>SMART BKK</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>BKK25</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E193" t="n">
+        <v>7</v>
+      </c>
+      <c r="F193" t="n">
+        <v>7</v>
+      </c>
+      <c r="G193" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>BKK27</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E194" t="n">
+        <v>50</v>
+      </c>
+      <c r="F194" t="n">
+        <v>50</v>
+      </c>
+      <c r="G194" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>BKK27</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E195" t="n">
+        <v>45</v>
+      </c>
+      <c r="F195" t="n">
+        <v>45</v>
+      </c>
+      <c r="G195" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>GATE IN</t>
+        </is>
+      </c>
+      <c r="E196" t="n">
+        <v>35</v>
+      </c>
+      <c r="F196" t="n">
+        <v>35</v>
+      </c>
+      <c r="G196" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>PW</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>LCHY5</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>GATE OUT</t>
+        </is>
+      </c>
+      <c r="E197" t="n">
+        <v>51</v>
+      </c>
+      <c r="F197" t="n">
+        <v>51</v>
+      </c>
+      <c r="G197" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G191"/>
+  <autoFilter ref="A1:G197"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Local TPSZ corrections file; C########## codes count as Agent; 24/10 PW fixes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gate-move-summary.xlsx
+++ b/docs/gate-move-summary.xlsx
@@ -21877,16 +21877,16 @@
         </is>
       </c>
       <c r="F390" t="n">
+        <v>15</v>
+      </c>
+      <c r="G390" t="n">
+        <v>0</v>
+      </c>
+      <c r="H390" t="n">
         <v>16</v>
       </c>
-      <c r="G390" t="n">
-        <v>0</v>
-      </c>
-      <c r="H390" t="n">
-        <v>18</v>
-      </c>
       <c r="I390" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J390" t="n">
         <v>0</v>
@@ -21904,7 +21904,7 @@
         <v>0</v>
       </c>
       <c r="O390" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="391">
@@ -21938,7 +21938,7 @@
         <v>0</v>
       </c>
       <c r="H391" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I391" t="n">
         <v>0</v>
@@ -21959,7 +21959,7 @@
         <v>0</v>
       </c>
       <c r="O391" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="392">

</xml_diff>

<commit_message>
Update 26/10/2026 (BC 0804, 10-26-GA2): all match
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gate-move-summary.xlsx
+++ b/docs/gate-move-summary.xlsx
@@ -22433,7 +22433,7 @@
         <v>0</v>
       </c>
       <c r="H400" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I400" t="n">
         <v>0</v>
@@ -22454,7 +22454,7 @@
         <v>0</v>
       </c>
       <c r="O400" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="401">
@@ -29015,13 +29015,13 @@
         </is>
       </c>
       <c r="E201" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F201" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="G201" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="202">
@@ -29192,10 +29192,10 @@
         <v>65</v>
       </c>
       <c r="F207" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G207" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>